<commit_message>
Marketing Page Rework & New Logos
</commit_message>
<xml_diff>
--- a/docs/INPROFIC_Q4_2026_Content_Calendar.xlsx
+++ b/docs/INPROFIC_Q4_2026_Content_Calendar.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Summary" sheetId="1" r:id="Rf3b1c7c3fc7c4468"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendar" sheetId="2" r:id="R5b98cc90a609405d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Catalog" sheetId="3" r:id="Reef88c99f82c4919"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Guide" sheetId="4" r:id="R24d94b6fe1374265"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Summary" sheetId="1" r:id="Rd516e238f33f4c9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendar" sheetId="2" r:id="R51b74aa8e87c4e32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Catalog" sheetId="3" r:id="R262b37945c0e4d55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Guide" sheetId="4" r:id="Raca407a3e62a46a2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -320,7 +320,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureCatalog" displayName="FeatureCatalog" ref="A1:G42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureCatalog" displayName="FeatureCatalog" ref="A1:G43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Feature ID"/>
     <x:tableColumn id="2" name="Capability"/>
@@ -586,7 +586,7 @@
       </x:c>
       <x:c r="B5" t="n">
         <x:f>COUNTA('Feature Catalog'!A2:A200)</x:f>
-        <x:v>41</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D5" s="13" t="str">
         <x:v>8–31 October</x:v>
@@ -601,7 +601,7 @@
       </x:c>
       <x:c r="B6" t="n">
         <x:f>COUNTIF('Feature Catalog'!F2:F200,"NEW")</x:f>
-        <x:v>11</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D6" s="13" t="str">
         <x:v>November</x:v>
@@ -692,7 +692,7 @@
         <x:v>Persistent stock alerts inside the shared operations tray</x:v>
       </x:c>
       <x:c r="B14" s="13" t="str">
-        <x:v>Raw-material and finished-good warning/low conditions open in separate Inventory tabs inside the movable tray, keep per-user snooze/re-alert timing, repeat a chosen INPROFIC tune in the foreground, and continue due reminders through Web Push when the app is backgrounded or closed.</x:v>
+        <x:v>Raw-material and finished-good warning/low conditions open in separate Inventory tabs inside the movable tray, keep per-user snooze/re-alert timing, can use synthesized alerts or eight bundled audio chimes, and continue due reminders through Web Push when the app is backgrounded or closed.</x:v>
       </x:c>
       <x:c r="C14" s="34" t="n">
         <x:v>46285</x:v>
@@ -725,7 +725,7 @@
         <x:v>Shared realtime Commerce, payment and delivery alert tray</x:v>
       </x:c>
       <x:c r="B17" s="13" t="str">
-        <x:v>Commerce, payment and Delivery alerts share one movable tray with Inventory without sharing read state; five selectable foreground tunes and configurable repeats keep unread work—including direct Transfer verification—hard to miss, while durable Web Push continues due reminders in the background.</x:v>
+        <x:v>Commerce, payment and Delivery alerts share one movable tray with Inventory without sharing read state; synthesized tones plus eight bundled audio chimes and configurable repeats keep unread work—including direct Transfer verification—hard to miss, while durable Web Push continues due reminders in the background.</x:v>
       </x:c>
       <x:c r="C17" s="34" t="n">
         <x:v>46285</x:v>
@@ -733,21 +733,21 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="32" t="str">
-        <x:v>Founder-controlled third-party integration availability</x:v>
+        <x:v>Founder-controlled subscription plans &amp; trial policy</x:v>
       </x:c>
       <x:c r="B18" s="13" t="str">
-        <x:v>Optional provider connectors can be hidden and execution-blocked platform-wide without deleting tenant credentials or history; businesses still activate their own approved provider accounts only after configuration.</x:v>
+        <x:v>Control plan pricing, module entitlements, the general free-trial duration and per-business founder trial extensions without deleting tenant history or overlapping active paid/lifetime access.</x:v>
       </x:c>
       <x:c r="C18" s="34" t="n">
-        <x:v>46285</x:v>
+        <x:v>46286</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="32" t="str">
-        <x:v>Plan-upgrade data continuity</x:v>
+        <x:v>Founder-controlled third-party integration availability</x:v>
       </x:c>
       <x:c r="B19" s="13" t="str">
-        <x:v>Hidden interconnected modules do not stop required back-office synchronization, so upgrades reveal already-complete records.</x:v>
+        <x:v>Optional provider connectors can be hidden and execution-blocked platform-wide without deleting tenant credentials or history; businesses still activate their own approved provider accounts only after configuration.</x:v>
       </x:c>
       <x:c r="C19" s="34" t="n">
         <x:v>46285</x:v>
@@ -758,7 +758,7 @@
         <x:v>Maintenance rule: whenever a user-visible INPROFIC capability is added or materially changed, update docs/feature_marketing_catalog.json and run scripts/generate_marketing_calendar.py. The CSV, Markdown and Excel outputs are regenerated together; new additions remain visibly marked ✨ NEW.</x:v>
       </x:c>
       <x:c r="B20" s="41" t="str">
-        <x:v>Physical Store/direct pricing stays inside the staff POS, while hosted/headless commerce exposes Online plus Distribution/Bulk and INPROFIC enforces the chosen channel and minimum quantity server-side.</x:v>
+        <x:v>Hidden interconnected modules do not stop required back-office synchronization, so upgrades reveal already-complete records.</x:v>
       </x:c>
       <x:c r="C20" s="42" t="n">
         <x:v>46285</x:v>
@@ -771,10 +771,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32" t="str">
-        <x:v>Standard portions, composed products and Bulk Packs</x:v>
+        <x:v>Surface-safe Online, POS and Distribution pricing</x:v>
       </x:c>
       <x:c r="B21" s="13" t="str">
-        <x:v>Keep production in base units such as scoops/pieces/ml while customers buy plates, servings, bowls, cartons or other packs; show customer-safe package contents and preserve private yield conversions.</x:v>
+        <x:v>Physical Store/direct pricing stays inside the staff POS, while hosted/headless commerce exposes Online plus Distribution/Bulk and INPROFIC enforces the chosen channel and minimum quantity server-side.</x:v>
       </x:c>
       <x:c r="C21" s="34" t="n">
         <x:v>46285</x:v>
@@ -782,10 +782,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="32" t="str">
-        <x:v>Founder product and lead analytics</x:v>
+        <x:v>Standard portions, composed products and Bulk Packs</x:v>
       </x:c>
       <x:c r="B22" s="13" t="str">
-        <x:v>Track first-party signup leads, completed registrations, logins, subscription milestones and throttled module usage in Founder Console without recording passwords, payment secrets or arbitrary clickstreams.</x:v>
+        <x:v>Keep production in base units such as scoops/pieces/ml while customers buy plates, servings, bowls, cartons or other packs; show customer-safe package contents and preserve private yield conversions.</x:v>
       </x:c>
       <x:c r="C22" s="34" t="n">
         <x:v>46285</x:v>
@@ -793,10 +793,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="32" t="str">
-        <x:v>Animated, consistent form validation across INPROFIC</x:v>
+        <x:v>Founder product and lead analytics</x:v>
       </x:c>
       <x:c r="B23" s="13" t="str">
-        <x:v>HTML5 and Django validation share animated field states, contextual SVG affordances, accessible feedback and consistent toggle switches; dynamic rows inherit the same behavior.</x:v>
+        <x:v>Track first-party signup leads, completed registrations, logins, subscription milestones and throttled module usage in Founder Console without recording passwords, payment secrets or arbitrary clickstreams.</x:v>
       </x:c>
       <x:c r="C23" s="34" t="n">
         <x:v>46285</x:v>
@@ -804,13 +804,35 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="str">
-        <x:v>Channel-aware plain and add-on product options</x:v>
+        <x:v>Animated, consistent form validation across INPROFIC</x:v>
       </x:c>
       <x:c r="B24" s="13" t="str">
-        <x:v>Offer Extra Jollof, Single Chicken, bottles, pieces or other plain portions from the same Finished Good stock and recipe with independent Physical Store, Online and Bulk/Distribution availability and pricing.</x:v>
+        <x:v>HTML5 and Django validation share animated field states, contextual SVG affordances, accessible feedback and consistent toggle switches; dynamic rows inherit the same behavior.</x:v>
       </x:c>
       <x:c r="C24" s="34" t="n">
         <x:v>46285</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="32" t="str">
+        <x:v>Channel-aware plain and add-on product options</x:v>
+      </x:c>
+      <x:c r="B25" s="13" t="str">
+        <x:v>Offer Extra Jollof, Single Chicken, bottles, pieces or other plain portions from the same Finished Good stock and recipe with independent Physical Store, Online and Bulk/Distribution availability and pricing.</x:v>
+      </x:c>
+      <x:c r="C25" s="34" t="n">
+        <x:v>46285</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="32" t="str">
+        <x:v>Interactive product demos</x:v>
+      </x:c>
+      <x:c r="B26" s="13" t="str">
+        <x:v>The marketing site provides a vertical-aware click-through workflow plus module-card flip previews and a detailed storefront-to-fulfilment flow.</x:v>
+      </x:c>
+      <x:c r="C26" s="34" t="n">
+        <x:v>46286</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1563,7 +1585,7 @@
         <x:v>✨ NEW — Persistent stock alerts inside the shared operations tray: what changes when this is handled inside one connected system?</x:v>
       </x:c>
       <x:c r="O11" s="13" t="str">
-        <x:v>Show exactly what the feature does and the workflow it replaces. Proof point: Raw-material and finished-good warning/low conditions open in separate Inventory tabs inside the movable tray, keep per-user snooze/re-alert timing, repeat a chosen INPROFIC tune in the foreground, and continue due reminders through Web Push when the app is backgrounded or closed.</x:v>
+        <x:v>Show exactly what the feature does and the workflow it replaces. Proof point: Raw-material and finished-good warning/low conditions open in separate Inventory tabs inside the movable tray, keep per-user snooze/re-alert timing, can use synthesized alerts or eight bundled audio chimes, and continue due reminders through Web Push when the app is backgrounded or closed.</x:v>
       </x:c>
       <x:c r="P11" s="13" t="str">
         <x:v>See how it works</x:v>
@@ -1819,7 +1841,7 @@
         <x:v>Wholesale and retail stock-first workflows: what changes when this is handled inside one connected system?</x:v>
       </x:c>
       <x:c r="O15" s="13" t="str">
-        <x:v>Show exactly what the feature does and the workflow it replaces. Proof point: Procure and sell resale products without forcing them through Production.</x:v>
+        <x:v>Show exactly what the feature does and the workflow it replaces. Proof point: Wholesale and retail use procurement-first stock-product forms and supporting-supply controls without production-only recipe, batch or base-material fields.</x:v>
       </x:c>
       <x:c r="P15" s="13" t="str">
         <x:v>See how it works</x:v>
@@ -2961,7 +2983,7 @@
         <x:v>Still solving this manually? ✨ NEW — Shared realtime Commerce, payment and delivery alert tray keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O33" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Commerce, payment and Delivery alerts share one movable tray with Inventory without sharing read state; five selectable foreground tunes and configurable repeats keep unread work—including direct Transfer verification—hard to miss, while durable Web Push continues due reminders in the background.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Commerce, payment and Delivery alerts share one movable tray with Inventory without sharing read state; synthesized tones plus eight bundled audio chimes and configurable repeats keep unread work—including direct Transfer verification—hard to miss, while durable Web Push continues due reminders in the background.</x:v>
       </x:c>
       <x:c r="P33" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
@@ -3322,7 +3344,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H39" s="13" t="str">
-        <x:v>Founder-controlled subscription plans</x:v>
+        <x:v>✨ NEW — Founder-controlled subscription plans &amp; trial policy</x:v>
       </x:c>
       <x:c r="I39" s="13" t="str">
         <x:v>Problem → workflow</x:v>
@@ -3340,22 +3362,26 @@
         <x:v>INPROFIC operators and plan-managed tenants</x:v>
       </x:c>
       <x:c r="N39" s="13" t="str">
-        <x:v>Still solving this manually? Founder-controlled subscription plans keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
+        <x:v>Still solving this manually? ✨ NEW — Founder-controlled subscription plans &amp; trial policy keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O39" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Control plan pricing, module entitlements and commercial access without deleting tenant history.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Control plan pricing, module entitlements, the general free-trial duration and per-business founder trial extensions without deleting tenant history or overlapping active paid/lifetime access.</x:v>
       </x:c>
       <x:c r="P39" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
       </x:c>
       <x:c r="Q39" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Founder-controlled subscription plans. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
-      </x:c>
-      <x:c r="R39" s="13" t="str"/>
+        <x:v>Use a real INPROFIC screen/demo for Founder-controlled subscription plans &amp; trial policy. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+      </x:c>
+      <x:c r="R39" s="13" t="str">
+        <x:v>NEW</x:v>
+      </x:c>
       <x:c r="S39" s="13" t="str">
         <x:v>subscriptions</x:v>
       </x:c>
-      <x:c r="T39" s="34" t="str"/>
+      <x:c r="T39" s="34" t="n">
+        <x:v>46286</x:v>
+      </x:c>
       <x:c r="U39" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -3666,7 +3692,7 @@
         <x:v>Still solving this manually? Guided system onboarding keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O44" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: A replayable module-aware tour helps staff learn the workspace without developer terminology.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: A replayable tenant-aware tour keeps the original animated guide and adds a second module-specific preview that reflects the business vertical.</x:v>
       </x:c>
       <x:c r="P44" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
@@ -4031,7 +4057,7 @@
         <x:v>Week 7</x:v>
       </x:c>
       <x:c r="D50" s="13" t="str">
-        <x:v>operations</x:v>
+        <x:v>experience</x:v>
       </x:c>
       <x:c r="E50" s="13" t="str">
         <x:v>Screen / workflow demo</x:v>
@@ -4043,7 +4069,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H50" s="13" t="str">
-        <x:v>Inventory with purchase-to-usage units</x:v>
+        <x:v>✨ NEW — Interactive product demos</x:v>
       </x:c>
       <x:c r="I50" s="13" t="str">
         <x:v>Problem → workflow</x:v>
@@ -4058,25 +4084,29 @@
         <x:v>Instagram, Facebook, LinkedIn</x:v>
       </x:c>
       <x:c r="M50" s="13" t="str">
-        <x:v>owners, storekeepers, production teams</x:v>
+        <x:v>prospective businesses exploring INPROFIC</x:v>
       </x:c>
       <x:c r="N50" s="13" t="str">
-        <x:v>Still solving this manually? Inventory with purchase-to-usage units keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
+        <x:v>Still solving this manually? ✨ NEW — Interactive product demos keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O50" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Buy in packs or bags while stock and recipes stay accurate in the unit actually consumed.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: The marketing site provides a vertical-aware click-through workflow plus module-card flip previews and a detailed storefront-to-fulfilment flow.</x:v>
       </x:c>
       <x:c r="P50" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
       </x:c>
       <x:c r="Q50" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Inventory with purchase-to-usage units. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
-      </x:c>
-      <x:c r="R50" s="13" t="str"/>
+        <x:v>Use a real INPROFIC screen/demo for Interactive product demos. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+      </x:c>
+      <x:c r="R50" s="13" t="str">
+        <x:v>NEW</x:v>
+      </x:c>
       <x:c r="S50" s="13" t="str">
-        <x:v>inventory-units</x:v>
-      </x:c>
-      <x:c r="T50" s="34" t="str"/>
+        <x:v>interactive-product-demos</x:v>
+      </x:c>
+      <x:c r="T50" s="34" t="n">
+        <x:v>46286</x:v>
+      </x:c>
       <x:c r="U50" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -4094,7 +4124,7 @@
         <x:v>Week 8</x:v>
       </x:c>
       <x:c r="D51" s="13" t="str">
-        <x:v>experience</x:v>
+        <x:v>operations</x:v>
       </x:c>
       <x:c r="E51" s="13" t="str">
         <x:v>Connected-system handoff</x:v>
@@ -4106,7 +4136,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H51" s="13" t="str">
-        <x:v>Dashboard search and operating insights</x:v>
+        <x:v>Inventory with purchase-to-usage units</x:v>
       </x:c>
       <x:c r="I51" s="13" t="str">
         <x:v>Problem → workflow</x:v>
@@ -4121,23 +4151,23 @@
         <x:v>Instagram, Facebook</x:v>
       </x:c>
       <x:c r="M51" s="13" t="str">
-        <x:v>owners and managers</x:v>
+        <x:v>owners, storekeepers, production teams</x:v>
       </x:c>
       <x:c r="N51" s="13" t="str">
-        <x:v>Still solving this manually? Dashboard search and operating insights keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
+        <x:v>Still solving this manually? Inventory with purchase-to-usage units keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O51" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Search key business records quickly and review stock, commercial and period signals from one operating dashboard.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Buy in packs or bags while stock and recipes stay accurate in the unit actually consumed.</x:v>
       </x:c>
       <x:c r="P51" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
       </x:c>
       <x:c r="Q51" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Dashboard search and operating insights. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Inventory with purchase-to-usage units. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R51" s="13" t="str"/>
       <x:c r="S51" s="13" t="str">
-        <x:v>dashboard-insights</x:v>
+        <x:v>inventory-units</x:v>
       </x:c>
       <x:c r="T51" s="34" t="str"/>
       <x:c r="U51" s="13" t="str">
@@ -4157,7 +4187,7 @@
         <x:v>Week 8</x:v>
       </x:c>
       <x:c r="D52" s="13" t="str">
-        <x:v>operations</x:v>
+        <x:v>experience</x:v>
       </x:c>
       <x:c r="E52" s="13" t="str">
         <x:v>Control / verification</x:v>
@@ -4169,7 +4199,7 @@
         <x:v>Consideration</x:v>
       </x:c>
       <x:c r="H52" s="13" t="str">
-        <x:v>✨ NEW — Persistent stock alerts inside the shared operations tray</x:v>
+        <x:v>Dashboard search and operating insights</x:v>
       </x:c>
       <x:c r="I52" s="13" t="str">
         <x:v>Problem → workflow</x:v>
@@ -4184,29 +4214,25 @@
         <x:v>Instagram, LinkedIn</x:v>
       </x:c>
       <x:c r="M52" s="13" t="str">
-        <x:v>owners, storekeepers, managers</x:v>
+        <x:v>owners and managers</x:v>
       </x:c>
       <x:c r="N52" s="13" t="str">
-        <x:v>Still solving this manually? ✨ NEW — Persistent stock alerts inside the shared operations tray keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
+        <x:v>Still solving this manually? Dashboard search and operating insights keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O52" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Raw-material and finished-good warning/low conditions open in separate Inventory tabs inside the movable tray, keep per-user snooze/re-alert timing, repeat a chosen INPROFIC tune in the foreground, and continue due reminders through Web Push when the app is backgrounded or closed.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Search key business records quickly and review stock, commercial and period signals from one operating dashboard.</x:v>
       </x:c>
       <x:c r="P52" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
       </x:c>
       <x:c r="Q52" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Persistent stock alerts inside the shared operations tray. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
-      </x:c>
-      <x:c r="R52" s="13" t="str">
-        <x:v>NEW</x:v>
-      </x:c>
+        <x:v>Use a real INPROFIC screen/demo for Dashboard search and operating insights. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+      </x:c>
+      <x:c r="R52" s="13" t="str"/>
       <x:c r="S52" s="13" t="str">
-        <x:v>stock-alerts</x:v>
-      </x:c>
-      <x:c r="T52" s="34" t="n">
-        <x:v>46285</x:v>
-      </x:c>
+        <x:v>dashboard-insights</x:v>
+      </x:c>
+      <x:c r="T52" s="34" t="str"/>
       <x:c r="U52" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -4236,7 +4262,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H53" s="13" t="str">
-        <x:v>Business-defined product categories</x:v>
+        <x:v>✨ NEW — Persistent stock alerts inside the shared operations tray</x:v>
       </x:c>
       <x:c r="I53" s="13" t="str">
         <x:v>Problem → workflow</x:v>
@@ -4251,25 +4277,29 @@
         <x:v>LinkedIn, Facebook</x:v>
       </x:c>
       <x:c r="M53" s="13" t="str">
-        <x:v>retail, restaurant, bakery and wholesale teams</x:v>
+        <x:v>owners, storekeepers, managers</x:v>
       </x:c>
       <x:c r="N53" s="13" t="str">
-        <x:v>Still solving this manually? Business-defined product categories keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
+        <x:v>Still solving this manually? ✨ NEW — Persistent stock alerts inside the shared operations tray keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O53" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Organize sellable products independently of whether they are made in-house or purchased for resale.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Raw-material and finished-good warning/low conditions open in separate Inventory tabs inside the movable tray, keep per-user snooze/re-alert timing, can use synthesized alerts or eight bundled audio chimes, and continue due reminders through Web Push when the app is backgrounded or closed.</x:v>
       </x:c>
       <x:c r="P53" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
       </x:c>
       <x:c r="Q53" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Business-defined product categories. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
-      </x:c>
-      <x:c r="R53" s="13" t="str"/>
+        <x:v>Use a real INPROFIC screen/demo for Persistent stock alerts inside the shared operations tray. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+      </x:c>
+      <x:c r="R53" s="13" t="str">
+        <x:v>NEW</x:v>
+      </x:c>
       <x:c r="S53" s="13" t="str">
-        <x:v>product-categories</x:v>
-      </x:c>
-      <x:c r="T53" s="34" t="str"/>
+        <x:v>stock-alerts</x:v>
+      </x:c>
+      <x:c r="T53" s="34" t="n">
+        <x:v>46285</x:v>
+      </x:c>
       <x:c r="U53" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -4299,7 +4329,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H54" s="13" t="str">
-        <x:v>Controlled measurement changes</x:v>
+        <x:v>Business-defined product categories</x:v>
       </x:c>
       <x:c r="I54" s="13" t="str">
         <x:v>Problem → workflow</x:v>
@@ -4314,23 +4344,23 @@
         <x:v>Instagram, TikTok</x:v>
       </x:c>
       <x:c r="M54" s="13" t="str">
-        <x:v>inventory and production managers</x:v>
+        <x:v>retail, restaurant, bakery and wholesale teams</x:v>
       </x:c>
       <x:c r="N54" s="13" t="str">
-        <x:v>Still solving this manually? Controlled measurement changes keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
+        <x:v>Still solving this manually? Business-defined product categories keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O54" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Convert live stock and recipe definitions without rewriting completed historical evidence.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Organize sellable products independently of whether they are made in-house or purchased for resale.</x:v>
       </x:c>
       <x:c r="P54" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
       </x:c>
       <x:c r="Q54" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Controlled measurement changes. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Business-defined product categories. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R54" s="13" t="str"/>
       <x:c r="S54" s="13" t="str">
-        <x:v>measurement-change</x:v>
+        <x:v>product-categories</x:v>
       </x:c>
       <x:c r="T54" s="34" t="str"/>
       <x:c r="U54" s="13" t="str">
@@ -4362,7 +4392,7 @@
         <x:v>Consideration</x:v>
       </x:c>
       <x:c r="H55" s="13" t="str">
-        <x:v>Procurement and receiving</x:v>
+        <x:v>Controlled measurement changes</x:v>
       </x:c>
       <x:c r="I55" s="13" t="str">
         <x:v>Problem → workflow</x:v>
@@ -4377,23 +4407,23 @@
         <x:v>Instagram Stories, Facebook Stories</x:v>
       </x:c>
       <x:c r="M55" s="13" t="str">
-        <x:v>procurement and store teams</x:v>
+        <x:v>inventory and production managers</x:v>
       </x:c>
       <x:c r="N55" s="13" t="str">
-        <x:v>Still solving this manually? Procurement and receiving keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
+        <x:v>Still solving this manually? Controlled measurement changes keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O55" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Receive purchase orders into stock with unit conversion and cost updates handled together.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Convert live stock and recipe definitions without rewriting completed historical evidence.</x:v>
       </x:c>
       <x:c r="P55" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
       </x:c>
       <x:c r="Q55" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Procurement and receiving. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Controlled measurement changes. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R55" s="13" t="str"/>
       <x:c r="S55" s="13" t="str">
-        <x:v>procurement</x:v>
+        <x:v>measurement-change</x:v>
       </x:c>
       <x:c r="T55" s="34" t="str"/>
       <x:c r="U55" s="13" t="str">
@@ -4425,7 +4455,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H56" s="13" t="str">
-        <x:v>Wholesale and retail stock-first workflows</x:v>
+        <x:v>Procurement and receiving</x:v>
       </x:c>
       <x:c r="I56" s="13" t="str">
         <x:v>Problem → workflow</x:v>
@@ -4440,23 +4470,23 @@
         <x:v>LinkedIn, Facebook</x:v>
       </x:c>
       <x:c r="M56" s="13" t="str">
-        <x:v>wholesalers and retailers</x:v>
+        <x:v>procurement and store teams</x:v>
       </x:c>
       <x:c r="N56" s="13" t="str">
-        <x:v>Still solving this manually? Wholesale and retail stock-first workflows keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
+        <x:v>Still solving this manually? Procurement and receiving keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O56" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Procure and sell resale products without forcing them through Production.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Receive purchase orders into stock with unit conversion and cost updates handled together.</x:v>
       </x:c>
       <x:c r="P56" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
       </x:c>
       <x:c r="Q56" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Wholesale and retail stock-first workflows. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Procurement and receiving. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R56" s="13" t="str"/>
       <x:c r="S56" s="13" t="str">
-        <x:v>wholesale-retail</x:v>
+        <x:v>procurement</x:v>
       </x:c>
       <x:c r="T56" s="34" t="str"/>
       <x:c r="U56" s="13" t="str">
@@ -4476,7 +4506,7 @@
         <x:v>Week 8</x:v>
       </x:c>
       <x:c r="D57" s="13" t="str">
-        <x:v>production</x:v>
+        <x:v>operations</x:v>
       </x:c>
       <x:c r="E57" s="13" t="str">
         <x:v>Screen / workflow demo</x:v>
@@ -4488,7 +4518,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H57" s="13" t="str">
-        <x:v>Production requests and orders</x:v>
+        <x:v>Wholesale and retail stock-first workflows</x:v>
       </x:c>
       <x:c r="I57" s="13" t="str">
         <x:v>Problem → workflow</x:v>
@@ -4503,23 +4533,23 @@
         <x:v>Instagram, Facebook, LinkedIn</x:v>
       </x:c>
       <x:c r="M57" s="13" t="str">
-        <x:v>production-led businesses</x:v>
+        <x:v>wholesalers and retailers</x:v>
       </x:c>
       <x:c r="N57" s="13" t="str">
-        <x:v>Still solving this manually? Production requests and orders keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
+        <x:v>Still solving this manually? Wholesale and retail stock-first workflows keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O57" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Plan output, release recipe materials transactionally and add completed output to finished stock.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Wholesale and retail use procurement-first stock-product forms and supporting-supply controls without production-only recipe, batch or base-material fields.</x:v>
       </x:c>
       <x:c r="P57" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
       </x:c>
       <x:c r="Q57" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Production requests and orders. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Wholesale and retail stock-first workflows. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R57" s="13" t="str"/>
       <x:c r="S57" s="13" t="str">
-        <x:v>production</x:v>
+        <x:v>wholesale-retail</x:v>
       </x:c>
       <x:c r="T57" s="34" t="str"/>
       <x:c r="U57" s="13" t="str">
@@ -4551,7 +4581,7 @@
         <x:v>Consideration</x:v>
       </x:c>
       <x:c r="H58" s="13" t="str">
-        <x:v>Shared Production Runs</x:v>
+        <x:v>Production requests and orders</x:v>
       </x:c>
       <x:c r="I58" s="13" t="str">
         <x:v>Problem → workflow</x:v>
@@ -4566,23 +4596,23 @@
         <x:v>Instagram, Facebook</x:v>
       </x:c>
       <x:c r="M58" s="13" t="str">
-        <x:v>production planners and managers</x:v>
+        <x:v>production-led businesses</x:v>
       </x:c>
       <x:c r="N58" s="13" t="str">
-        <x:v>Still solving this manually? Shared Production Runs keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
+        <x:v>Still solving this manually? Production requests and orders keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O58" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Coordinate multiple normal customer/restock orders into one combined material release without losing order-level attribution.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Plan output, release recipe materials transactionally and add completed output to finished stock.</x:v>
       </x:c>
       <x:c r="P58" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
       </x:c>
       <x:c r="Q58" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Shared Production Runs. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Production requests and orders. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R58" s="13" t="str"/>
       <x:c r="S58" s="13" t="str">
-        <x:v>shared-runs</x:v>
+        <x:v>production</x:v>
       </x:c>
       <x:c r="T58" s="34" t="str"/>
       <x:c r="U58" s="13" t="str">
@@ -4614,7 +4644,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H59" s="13" t="str">
-        <x:v>Batch yield, wastage and output tracking</x:v>
+        <x:v>Shared Production Runs</x:v>
       </x:c>
       <x:c r="I59" s="13" t="str">
         <x:v>Problem → workflow</x:v>
@@ -4629,23 +4659,23 @@
         <x:v>Instagram, LinkedIn</x:v>
       </x:c>
       <x:c r="M59" s="13" t="str">
-        <x:v>production teams</x:v>
+        <x:v>production planners and managers</x:v>
       </x:c>
       <x:c r="N59" s="13" t="str">
-        <x:v>Still solving this manually? Batch yield, wastage and output tracking keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
+        <x:v>Still solving this manually? Shared Production Runs keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O59" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Keep requested quantity, planned output, actual output and wastage distinct.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Coordinate multiple normal customer/restock orders into one combined material release without losing order-level attribution.</x:v>
       </x:c>
       <x:c r="P59" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
       </x:c>
       <x:c r="Q59" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Batch yield, wastage and output tracking. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Shared Production Runs. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R59" s="13" t="str"/>
       <x:c r="S59" s="13" t="str">
-        <x:v>batch-yield</x:v>
+        <x:v>shared-runs</x:v>
       </x:c>
       <x:c r="T59" s="34" t="str"/>
       <x:c r="U59" s="13" t="str">
@@ -4677,7 +4707,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H60" s="13" t="str">
-        <x:v>Offcut, surplus and shortage reconciliation</x:v>
+        <x:v>Batch yield, wastage and output tracking</x:v>
       </x:c>
       <x:c r="I60" s="13" t="str">
         <x:v>Problem → workflow</x:v>
@@ -4692,23 +4722,23 @@
         <x:v>LinkedIn, Facebook</x:v>
       </x:c>
       <x:c r="M60" s="13" t="str">
-        <x:v>production and sales managers</x:v>
+        <x:v>production teams</x:v>
       </x:c>
       <x:c r="N60" s="13" t="str">
-        <x:v>Still solving this manually? Offcut, surplus and shortage reconciliation keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
+        <x:v>Still solving this manually? Batch yield, wastage and output tracking keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O60" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Route usable surplus deliberately and reconcile customer shortages without duplicate sales or production events.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Keep requested quantity, planned output, actual output and wastage distinct.</x:v>
       </x:c>
       <x:c r="P60" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
       </x:c>
       <x:c r="Q60" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Offcut, surplus and shortage reconciliation. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Batch yield, wastage and output tracking. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R60" s="13" t="str"/>
       <x:c r="S60" s="13" t="str">
-        <x:v>offcuts-shortages</x:v>
+        <x:v>batch-yield</x:v>
       </x:c>
       <x:c r="T60" s="34" t="str"/>
       <x:c r="U60" s="13" t="str">
@@ -4728,7 +4758,7 @@
         <x:v>Week 9</x:v>
       </x:c>
       <x:c r="D61" s="13" t="str">
-        <x:v>sales</x:v>
+        <x:v>production</x:v>
       </x:c>
       <x:c r="E61" s="13" t="str">
         <x:v>Recap / CTA</x:v>
@@ -4740,7 +4770,7 @@
         <x:v>Consideration</x:v>
       </x:c>
       <x:c r="H61" s="13" t="str">
-        <x:v>Customer orders and sales</x:v>
+        <x:v>Offcut, surplus and shortage reconciliation</x:v>
       </x:c>
       <x:c r="I61" s="13" t="str">
         <x:v>Problem → workflow</x:v>
@@ -4755,23 +4785,23 @@
         <x:v>Instagram, TikTok</x:v>
       </x:c>
       <x:c r="M61" s="13" t="str">
-        <x:v>sales teams and owners</x:v>
+        <x:v>production and sales managers</x:v>
       </x:c>
       <x:c r="N61" s="13" t="str">
-        <x:v>Still solving this manually? Customer orders and sales keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
+        <x:v>Still solving this manually? Offcut, surplus and shortage reconciliation keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O61" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Handle walk-in and customer orders while preserving fulfilment and payment state separately.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Route usable surplus deliberately and reconcile customer shortages without duplicate sales or production events.</x:v>
       </x:c>
       <x:c r="P61" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
       </x:c>
       <x:c r="Q61" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Customer orders and sales. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Offcut, surplus and shortage reconciliation. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R61" s="13" t="str"/>
       <x:c r="S61" s="13" t="str">
-        <x:v>sales</x:v>
+        <x:v>offcuts-shortages</x:v>
       </x:c>
       <x:c r="T61" s="34" t="str"/>
       <x:c r="U61" s="13" t="str">
@@ -4803,7 +4833,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H62" s="13" t="str">
-        <x:v>Customer and channel pricing</x:v>
+        <x:v>Customer orders and sales</x:v>
       </x:c>
       <x:c r="I62" s="13" t="str">
         <x:v>Problem → workflow</x:v>
@@ -4818,23 +4848,23 @@
         <x:v>Instagram Stories, Facebook Stories</x:v>
       </x:c>
       <x:c r="M62" s="13" t="str">
-        <x:v>wholesale and distribution businesses</x:v>
+        <x:v>sales teams and owners</x:v>
       </x:c>
       <x:c r="N62" s="13" t="str">
-        <x:v>Still solving this manually? Customer and channel pricing keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
+        <x:v>Still solving this manually? Customer orders and sales keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O62" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Resolve customer-specific pricing before channel pricing, then fall back to the product default.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Handle walk-in and customer orders while preserving fulfilment and payment state separately.</x:v>
       </x:c>
       <x:c r="P62" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
       </x:c>
       <x:c r="Q62" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Customer and channel pricing. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Customer orders and sales. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R62" s="13" t="str"/>
       <x:c r="S62" s="13" t="str">
-        <x:v>customer-pricing</x:v>
+        <x:v>sales</x:v>
       </x:c>
       <x:c r="T62" s="34" t="str"/>
       <x:c r="U62" s="13" t="str">
@@ -4854,7 +4884,7 @@
         <x:v>Week 9</x:v>
       </x:c>
       <x:c r="D63" s="13" t="str">
-        <x:v>finance</x:v>
+        <x:v>sales</x:v>
       </x:c>
       <x:c r="E63" s="13" t="str">
         <x:v>How it works</x:v>
@@ -4866,7 +4896,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H63" s="13" t="str">
-        <x:v>Receivables, payables and partial settlement</x:v>
+        <x:v>Customer and channel pricing</x:v>
       </x:c>
       <x:c r="I63" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -4881,23 +4911,23 @@
         <x:v>LinkedIn, Facebook</x:v>
       </x:c>
       <x:c r="M63" s="13" t="str">
-        <x:v>owners and finance teams</x:v>
+        <x:v>wholesale and distribution businesses</x:v>
       </x:c>
       <x:c r="N63" s="13" t="str">
-        <x:v>Year-end control check: Receivables, payables and partial settlement gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Customer and channel pricing gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O63" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Track what is owed separately from real cash movement and support partial settlement without false paid states.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Resolve customer-specific pricing before channel pricing, then fall back to the product default.</x:v>
       </x:c>
       <x:c r="P63" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q63" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Receivables, payables and partial settlement. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Customer and channel pricing. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R63" s="13" t="str"/>
       <x:c r="S63" s="13" t="str">
-        <x:v>credit</x:v>
+        <x:v>customer-pricing</x:v>
       </x:c>
       <x:c r="T63" s="34" t="str"/>
       <x:c r="U63" s="13" t="str">
@@ -4929,7 +4959,7 @@
         <x:v>Consideration</x:v>
       </x:c>
       <x:c r="H64" s="13" t="str">
-        <x:v>Auditable cash and finance ledger</x:v>
+        <x:v>Receivables, payables and partial settlement</x:v>
       </x:c>
       <x:c r="I64" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -4944,23 +4974,23 @@
         <x:v>Instagram, Facebook, LinkedIn</x:v>
       </x:c>
       <x:c r="M64" s="13" t="str">
-        <x:v>finance teams and owners</x:v>
+        <x:v>owners and finance teams</x:v>
       </x:c>
       <x:c r="N64" s="13" t="str">
-        <x:v>Year-end control check: Auditable cash and finance ledger gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Receivables, payables and partial settlement gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O64" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Verified money movement posts to tenant-owned accounts with compensating reversals instead of destructive edits.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Track what is owed separately from real cash movement and support partial settlement without false paid states.</x:v>
       </x:c>
       <x:c r="P64" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q64" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Auditable cash and finance ledger. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Receivables, payables and partial settlement. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R64" s="13" t="str"/>
       <x:c r="S64" s="13" t="str">
-        <x:v>finance-ledger</x:v>
+        <x:v>credit</x:v>
       </x:c>
       <x:c r="T64" s="34" t="str"/>
       <x:c r="U64" s="13" t="str">
@@ -4992,7 +5022,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H65" s="13" t="str">
-        <x:v>Expenses and expense settlement</x:v>
+        <x:v>Auditable cash and finance ledger</x:v>
       </x:c>
       <x:c r="I65" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5007,23 +5037,23 @@
         <x:v>Instagram, Facebook</x:v>
       </x:c>
       <x:c r="M65" s="13" t="str">
-        <x:v>owners and finance teams</x:v>
+        <x:v>finance teams and owners</x:v>
       </x:c>
       <x:c r="N65" s="13" t="str">
-        <x:v>Year-end control check: Expenses and expense settlement gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Auditable cash and finance ledger gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O65" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Record business expenses, distinguish unpaid obligations from actual settlement, and feed paid amounts into the cash ledger.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Verified money movement posts to tenant-owned accounts with compensating reversals instead of destructive edits.</x:v>
       </x:c>
       <x:c r="P65" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q65" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Expenses and expense settlement. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Auditable cash and finance ledger. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R65" s="13" t="str"/>
       <x:c r="S65" s="13" t="str">
-        <x:v>expenses</x:v>
+        <x:v>finance-ledger</x:v>
       </x:c>
       <x:c r="T65" s="34" t="str"/>
       <x:c r="U65" s="13" t="str">
@@ -5043,7 +5073,7 @@
         <x:v>Week 10</x:v>
       </x:c>
       <x:c r="D66" s="13" t="str">
-        <x:v>commerce</x:v>
+        <x:v>finance</x:v>
       </x:c>
       <x:c r="E66" s="13" t="str">
         <x:v>Control / verification</x:v>
@@ -5055,7 +5085,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H66" s="13" t="str">
-        <x:v>Hosted storefront and Order Now</x:v>
+        <x:v>Expenses and expense settlement</x:v>
       </x:c>
       <x:c r="I66" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5070,23 +5100,23 @@
         <x:v>Instagram, LinkedIn</x:v>
       </x:c>
       <x:c r="M66" s="13" t="str">
-        <x:v>businesses selling online without a custom commerce stack</x:v>
+        <x:v>owners and finance teams</x:v>
       </x:c>
       <x:c r="N66" s="13" t="str">
-        <x:v>Year-end control check: Hosted storefront and Order Now gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Expenses and expense settlement gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O66" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Publish tenant products, take baskets and start payment-first checkout without creating premature operational records.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Record business expenses, distinguish unpaid obligations from actual settlement, and feed paid amounts into the cash ledger.</x:v>
       </x:c>
       <x:c r="P66" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q66" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Hosted storefront and Order Now. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Expenses and expense settlement. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R66" s="13" t="str"/>
       <x:c r="S66" s="13" t="str">
-        <x:v>commerce-storefront</x:v>
+        <x:v>expenses</x:v>
       </x:c>
       <x:c r="T66" s="34" t="str"/>
       <x:c r="U66" s="13" t="str">
@@ -5118,7 +5148,7 @@
         <x:v>Consideration</x:v>
       </x:c>
       <x:c r="H67" s="13" t="str">
-        <x:v>Headless Commerce API</x:v>
+        <x:v>Hosted storefront and Order Now</x:v>
       </x:c>
       <x:c r="I67" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5133,23 +5163,23 @@
         <x:v>LinkedIn, Facebook</x:v>
       </x:c>
       <x:c r="M67" s="13" t="str">
-        <x:v>businesses with custom websites or apps</x:v>
+        <x:v>businesses selling online without a custom commerce stack</x:v>
       </x:c>
       <x:c r="N67" s="13" t="str">
-        <x:v>Year-end control check: Headless Commerce API gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Hosted storefront and Order Now gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O67" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: External websites consume authoritative catalogue, checkout, payment, delivery and tracking endpoints while keys stay server-side; external pricing exposes Online and Distribution/Bulk only, never the in-premise Physical Store price.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Publish tenant products, take baskets and start payment-first checkout without creating premature operational records.</x:v>
       </x:c>
       <x:c r="P67" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q67" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Headless Commerce API. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Hosted storefront and Order Now. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R67" s="13" t="str"/>
       <x:c r="S67" s="13" t="str">
-        <x:v>headless-api</x:v>
+        <x:v>commerce-storefront</x:v>
       </x:c>
       <x:c r="T67" s="34" t="str"/>
       <x:c r="U67" s="13" t="str">
@@ -5181,7 +5211,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H68" s="13" t="str">
-        <x:v>Paystack and Monnify payments</x:v>
+        <x:v>Headless Commerce API</x:v>
       </x:c>
       <x:c r="I68" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5196,23 +5226,23 @@
         <x:v>Instagram, TikTok</x:v>
       </x:c>
       <x:c r="M68" s="13" t="str">
-        <x:v>online-selling businesses</x:v>
+        <x:v>businesses with custom websites or apps</x:v>
       </x:c>
       <x:c r="N68" s="13" t="str">
-        <x:v>Year-end control check: Paystack and Monnify payments gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Headless Commerce API gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O68" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Provider-backed checkout and instant transfer settle only after authoritative provider verification.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: External websites consume authoritative catalogue, checkout, payment, delivery and tracking endpoints while keys stay server-side; external pricing exposes Online and Distribution/Bulk only, never the in-premise Physical Store price.</x:v>
       </x:c>
       <x:c r="P68" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q68" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Paystack and Monnify payments. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Headless Commerce API. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R68" s="13" t="str"/>
       <x:c r="S68" s="13" t="str">
-        <x:v>gateway-payments</x:v>
+        <x:v>headless-api</x:v>
       </x:c>
       <x:c r="T68" s="34" t="str"/>
       <x:c r="U68" s="13" t="str">
@@ -5244,7 +5274,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H69" s="13" t="str">
-        <x:v>✨ NEW — Transfer without a payment gateway</x:v>
+        <x:v>Paystack and Monnify payments</x:v>
       </x:c>
       <x:c r="I69" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5259,29 +5289,25 @@
         <x:v>Instagram Stories, Facebook Stories</x:v>
       </x:c>
       <x:c r="M69" s="13" t="str">
-        <x:v>businesses that prefer direct bank transfer</x:v>
+        <x:v>online-selling businesses</x:v>
       </x:c>
       <x:c r="N69" s="13" t="str">
-        <x:v>Year-end control check: ✨ NEW — Transfer without a payment gateway gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Paystack and Monnify payments gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O69" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Show the business bank account, require customer payment proof externally, and keep payment pending until staff verifies the actual credit.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Provider-backed checkout and instant transfer settle only after authoritative provider verification.</x:v>
       </x:c>
       <x:c r="P69" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q69" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Transfer without a payment gateway. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
-      </x:c>
-      <x:c r="R69" s="13" t="str">
-        <x:v>NEW</x:v>
-      </x:c>
+        <x:v>Use a real INPROFIC screen/demo for Paystack and Monnify payments. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+      </x:c>
+      <x:c r="R69" s="13" t="str"/>
       <x:c r="S69" s="13" t="str">
-        <x:v>direct-transfer</x:v>
-      </x:c>
-      <x:c r="T69" s="34" t="n">
-        <x:v>46285</x:v>
-      </x:c>
+        <x:v>gateway-payments</x:v>
+      </x:c>
+      <x:c r="T69" s="34" t="str"/>
       <x:c r="U69" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -5311,7 +5337,7 @@
         <x:v>Consideration</x:v>
       </x:c>
       <x:c r="H70" s="13" t="str">
-        <x:v>In-premise POS</x:v>
+        <x:v>✨ NEW — Transfer without a payment gateway</x:v>
       </x:c>
       <x:c r="I70" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5326,25 +5352,29 @@
         <x:v>LinkedIn, Facebook</x:v>
       </x:c>
       <x:c r="M70" s="13" t="str">
-        <x:v>cashiers, stores, restaurants and walk-in operations</x:v>
+        <x:v>businesses that prefer direct bank transfer</x:v>
       </x:c>
       <x:c r="N70" s="13" t="str">
-        <x:v>Year-end control check: In-premise POS gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: ✨ NEW — Transfer without a payment gateway gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O70" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Staff can complete counter sales with Cash, direct Transfer or supported terminal payment without opening the wider workspace.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Show the business bank account, require customer payment proof externally, and keep payment pending until staff verifies the actual credit.</x:v>
       </x:c>
       <x:c r="P70" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q70" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for In-premise POS. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
-      </x:c>
-      <x:c r="R70" s="13" t="str"/>
+        <x:v>Use a real INPROFIC screen/demo for Transfer without a payment gateway. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+      </x:c>
+      <x:c r="R70" s="13" t="str">
+        <x:v>NEW</x:v>
+      </x:c>
       <x:c r="S70" s="13" t="str">
-        <x:v>pos</x:v>
-      </x:c>
-      <x:c r="T70" s="34" t="str"/>
+        <x:v>direct-transfer</x:v>
+      </x:c>
+      <x:c r="T70" s="34" t="n">
+        <x:v>46285</x:v>
+      </x:c>
       <x:c r="U70" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -5362,7 +5392,7 @@
         <x:v>Week 10</x:v>
       </x:c>
       <x:c r="D71" s="13" t="str">
-        <x:v>delivery</x:v>
+        <x:v>commerce</x:v>
       </x:c>
       <x:c r="E71" s="13" t="str">
         <x:v>Screen / workflow demo</x:v>
@@ -5374,7 +5404,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H71" s="13" t="str">
-        <x:v>Delivery quoting and hybrid routing</x:v>
+        <x:v>In-premise POS</x:v>
       </x:c>
       <x:c r="I71" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5389,23 +5419,23 @@
         <x:v>Instagram, Facebook, LinkedIn</x:v>
       </x:c>
       <x:c r="M71" s="13" t="str">
-        <x:v>businesses delivering customer orders</x:v>
+        <x:v>cashiers, stores, restaurants and walk-in operations</x:v>
       </x:c>
       <x:c r="N71" s="13" t="str">
-        <x:v>Year-end control check: Delivery quoting and hybrid routing gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: In-premise POS gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O71" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Quote from validated destinations before payment and switch between in-house and configured provider routing under tenant policy.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Staff can complete counter sales with Cash, direct Transfer or supported terminal payment without opening the wider workspace.</x:v>
       </x:c>
       <x:c r="P71" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q71" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Delivery quoting and hybrid routing. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for In-premise POS. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R71" s="13" t="str"/>
       <x:c r="S71" s="13" t="str">
-        <x:v>delivery</x:v>
+        <x:v>pos</x:v>
       </x:c>
       <x:c r="T71" s="34" t="str"/>
       <x:c r="U71" s="13" t="str">
@@ -5437,7 +5467,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H72" s="13" t="str">
-        <x:v>Mapped delivery areas and precise address validation</x:v>
+        <x:v>Delivery quoting and hybrid routing</x:v>
       </x:c>
       <x:c r="I72" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5452,23 +5482,23 @@
         <x:v>Instagram, Facebook</x:v>
       </x:c>
       <x:c r="M72" s="13" t="str">
-        <x:v>dispatch teams and online-selling businesses</x:v>
+        <x:v>businesses delivering customer orders</x:v>
       </x:c>
       <x:c r="N72" s="13" t="str">
-        <x:v>Year-end control check: Mapped delivery areas and precise address validation gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Delivery quoting and hybrid routing gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O72" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Define delivery coverage, locate typed addresses after a calm 2-second idle window, keep corrections from being overwritten by stale lookups, and fall back to a customer map pin before quoting delivery.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Quote from validated destinations before payment and switch between in-house and configured provider routing under tenant policy.</x:v>
       </x:c>
       <x:c r="P72" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q72" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Mapped delivery areas and precise address validation. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Delivery quoting and hybrid routing. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R72" s="13" t="str"/>
       <x:c r="S72" s="13" t="str">
-        <x:v>delivery-coverage</x:v>
+        <x:v>delivery</x:v>
       </x:c>
       <x:c r="T72" s="34" t="str"/>
       <x:c r="U72" s="13" t="str">
@@ -5500,7 +5530,7 @@
         <x:v>Consideration</x:v>
       </x:c>
       <x:c r="H73" s="13" t="str">
-        <x:v>✨ NEW — Provider-neutral delivery partner adapters</x:v>
+        <x:v>Mapped delivery areas and precise address validation</x:v>
       </x:c>
       <x:c r="I73" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5515,29 +5545,25 @@
         <x:v>Instagram, LinkedIn</x:v>
       </x:c>
       <x:c r="M73" s="13" t="str">
-        <x:v>businesses using in-house riders, couriers or external delivery partners</x:v>
+        <x:v>dispatch teams and online-selling businesses</x:v>
       </x:c>
       <x:c r="N73" s="13" t="str">
-        <x:v>Year-end control check: ✨ NEW — Provider-neutral delivery partner adapters gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Mapped delivery areas and precise address validation gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O73" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Keep INPROFIC in control of delivery pricing, routing and tracking while any courier stays manual or connects through a normalized dispatch/status adapter; optional built-in providers remain separately governed.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Define delivery coverage, locate typed addresses after a calm 2-second idle window, keep corrections from being overwritten by stale lookups, and fall back to a customer map pin before quoting delivery.</x:v>
       </x:c>
       <x:c r="P73" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q73" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Provider-neutral delivery partner adapters. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
-      </x:c>
-      <x:c r="R73" s="13" t="str">
-        <x:v>NEW</x:v>
-      </x:c>
+        <x:v>Use a real INPROFIC screen/demo for Mapped delivery areas and precise address validation. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+      </x:c>
+      <x:c r="R73" s="13" t="str"/>
       <x:c r="S73" s="13" t="str">
-        <x:v>glovo-provider</x:v>
-      </x:c>
-      <x:c r="T73" s="34" t="n">
-        <x:v>46285</x:v>
-      </x:c>
+        <x:v>delivery-coverage</x:v>
+      </x:c>
+      <x:c r="T73" s="34" t="str"/>
       <x:c r="U73" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -5567,7 +5593,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H74" s="13" t="str">
-        <x:v>✨ NEW — Shared realtime Commerce, payment and delivery alert tray</x:v>
+        <x:v>✨ NEW — Provider-neutral delivery partner adapters</x:v>
       </x:c>
       <x:c r="I74" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5582,25 +5608,25 @@
         <x:v>LinkedIn, Facebook</x:v>
       </x:c>
       <x:c r="M74" s="13" t="str">
-        <x:v>dispatchers, managers and riders</x:v>
+        <x:v>businesses using in-house riders, couriers or external delivery partners</x:v>
       </x:c>
       <x:c r="N74" s="13" t="str">
-        <x:v>Year-end control check: ✨ NEW — Shared realtime Commerce, payment and delivery alert tray gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: ✨ NEW — Provider-neutral delivery partner adapters gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O74" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Commerce, payment and Delivery alerts share one movable tray with Inventory without sharing read state; five selectable foreground tunes and configurable repeats keep unread work—including direct Transfer verification—hard to miss, while durable Web Push continues due reminders in the background.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Keep INPROFIC in control of delivery pricing, routing and tracking while any courier stays manual or connects through a normalized dispatch/status adapter; optional built-in providers remain separately governed.</x:v>
       </x:c>
       <x:c r="P74" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q74" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Shared realtime Commerce, payment and delivery alert tray. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Provider-neutral delivery partner adapters. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R74" s="13" t="str">
         <x:v>NEW</x:v>
       </x:c>
       <x:c r="S74" s="13" t="str">
-        <x:v>delivery-notifications</x:v>
+        <x:v>glovo-provider</x:v>
       </x:c>
       <x:c r="T74" s="34" t="n">
         <x:v>46285</x:v>
@@ -5634,7 +5660,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H75" s="13" t="str">
-        <x:v>Delivery Rider workspace</x:v>
+        <x:v>✨ NEW — Shared realtime Commerce, payment and delivery alert tray</x:v>
       </x:c>
       <x:c r="I75" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5649,25 +5675,29 @@
         <x:v>Instagram, TikTok</x:v>
       </x:c>
       <x:c r="M75" s="13" t="str">
-        <x:v>in-house riders and dispatch teams</x:v>
+        <x:v>dispatchers, managers and riders</x:v>
       </x:c>
       <x:c r="N75" s="13" t="str">
-        <x:v>Year-end control check: Delivery Rider workspace gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: ✨ NEW — Shared realtime Commerce, payment and delivery alert tray gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O75" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Riders see only assigned deliveries, allowed status actions and proof-of-delivery; admins control the rider alert tune/repeat policy and riders can enroll their own device for background Web Push.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Commerce, payment and Delivery alerts share one movable tray with Inventory without sharing read state; synthesized tones plus eight bundled audio chimes and configurable repeats keep unread work—including direct Transfer verification—hard to miss, while durable Web Push continues due reminders in the background.</x:v>
       </x:c>
       <x:c r="P75" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q75" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Delivery Rider workspace. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
-      </x:c>
-      <x:c r="R75" s="13" t="str"/>
+        <x:v>Use a real INPROFIC screen/demo for Shared realtime Commerce, payment and delivery alert tray. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+      </x:c>
+      <x:c r="R75" s="13" t="str">
+        <x:v>NEW</x:v>
+      </x:c>
       <x:c r="S75" s="13" t="str">
-        <x:v>rider</x:v>
-      </x:c>
-      <x:c r="T75" s="34" t="str"/>
+        <x:v>delivery-notifications</x:v>
+      </x:c>
+      <x:c r="T75" s="34" t="n">
+        <x:v>46285</x:v>
+      </x:c>
       <x:c r="U75" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -5685,7 +5715,7 @@
         <x:v>Week 11</x:v>
       </x:c>
       <x:c r="D76" s="13" t="str">
-        <x:v>commerce</x:v>
+        <x:v>delivery</x:v>
       </x:c>
       <x:c r="E76" s="13" t="str">
         <x:v>Problem / pain point</x:v>
@@ -5697,7 +5727,7 @@
         <x:v>Consideration</x:v>
       </x:c>
       <x:c r="H76" s="13" t="str">
-        <x:v>Storefront customer profiles and tracking</x:v>
+        <x:v>Delivery Rider workspace</x:v>
       </x:c>
       <x:c r="I76" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5712,23 +5742,23 @@
         <x:v>Instagram Stories, Facebook Stories</x:v>
       </x:c>
       <x:c r="M76" s="13" t="str">
-        <x:v>repeat online customers</x:v>
+        <x:v>in-house riders and dispatch teams</x:v>
       </x:c>
       <x:c r="N76" s="13" t="str">
-        <x:v>Year-end control check: Storefront customer profiles and tracking gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Delivery Rider workspace gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O76" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Optional tenant-scoped customer accounts save contact details and purchase history while guest checkout remains available.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Riders see only assigned deliveries, allowed status actions and proof-of-delivery; admins control the rider alert tune/repeat policy and riders can enroll their own device for background Web Push.</x:v>
       </x:c>
       <x:c r="P76" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q76" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Storefront customer profiles and tracking. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Delivery Rider workspace. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R76" s="13" t="str"/>
       <x:c r="S76" s="13" t="str">
-        <x:v>customer-profiles</x:v>
+        <x:v>rider</x:v>
       </x:c>
       <x:c r="T76" s="34" t="str"/>
       <x:c r="U76" s="13" t="str">
@@ -5748,7 +5778,7 @@
         <x:v>Week 11</x:v>
       </x:c>
       <x:c r="D77" s="13" t="str">
-        <x:v>governance</x:v>
+        <x:v>commerce</x:v>
       </x:c>
       <x:c r="E77" s="13" t="str">
         <x:v>How it works</x:v>
@@ -5760,7 +5790,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H77" s="13" t="str">
-        <x:v>Audit Workspace</x:v>
+        <x:v>Storefront customer profiles and tracking</x:v>
       </x:c>
       <x:c r="I77" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5775,23 +5805,23 @@
         <x:v>LinkedIn, Facebook</x:v>
       </x:c>
       <x:c r="M77" s="13" t="str">
-        <x:v>owners, finance teams and external auditors</x:v>
+        <x:v>repeat online customers</x:v>
       </x:c>
       <x:c r="N77" s="13" t="str">
-        <x:v>Year-end control check: Audit Workspace gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Storefront customer profiles and tracking gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O77" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Provide plan-gated read-only cross-module evidence review with auditor queries, flags and response tracking.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Optional tenant-scoped customer accounts save contact details and purchase history while guest checkout remains available.</x:v>
       </x:c>
       <x:c r="P77" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q77" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Audit Workspace. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Storefront customer profiles and tracking. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R77" s="13" t="str"/>
       <x:c r="S77" s="13" t="str">
-        <x:v>audit</x:v>
+        <x:v>customer-profiles</x:v>
       </x:c>
       <x:c r="T77" s="34" t="str"/>
       <x:c r="U77" s="13" t="str">
@@ -5823,7 +5853,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H78" s="13" t="str">
-        <x:v>Role and per-user permissions</x:v>
+        <x:v>Audit Workspace</x:v>
       </x:c>
       <x:c r="I78" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5838,23 +5868,23 @@
         <x:v>Instagram, Facebook, LinkedIn</x:v>
       </x:c>
       <x:c r="M78" s="13" t="str">
-        <x:v>growing teams</x:v>
+        <x:v>owners, finance teams and external auditors</x:v>
       </x:c>
       <x:c r="N78" s="13" t="str">
-        <x:v>Year-end control check: Role and per-user permissions gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Audit Workspace gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O78" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Give staff only the workspaces and actions they need while business-level entitlements remain the ceiling.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Provide plan-gated read-only cross-module evidence review with auditor queries, flags and response tracking.</x:v>
       </x:c>
       <x:c r="P78" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q78" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Role and per-user permissions. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Audit Workspace. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R78" s="13" t="str"/>
       <x:c r="S78" s="13" t="str">
-        <x:v>roles</x:v>
+        <x:v>audit</x:v>
       </x:c>
       <x:c r="T78" s="34" t="str"/>
       <x:c r="U78" s="13" t="str">
@@ -5874,7 +5904,7 @@
         <x:v>Week 12</x:v>
       </x:c>
       <x:c r="D79" s="13" t="str">
-        <x:v>experience</x:v>
+        <x:v>governance</x:v>
       </x:c>
       <x:c r="E79" s="13" t="str">
         <x:v>Connected-system handoff</x:v>
@@ -5886,7 +5916,7 @@
         <x:v>Consideration</x:v>
       </x:c>
       <x:c r="H79" s="13" t="str">
-        <x:v>Tenant branding and workspace appearance</x:v>
+        <x:v>Role and per-user permissions</x:v>
       </x:c>
       <x:c r="I79" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5901,23 +5931,23 @@
         <x:v>Instagram, Facebook</x:v>
       </x:c>
       <x:c r="M79" s="13" t="str">
-        <x:v>business owners and teams</x:v>
+        <x:v>growing teams</x:v>
       </x:c>
       <x:c r="N79" s="13" t="str">
-        <x:v>Year-end control check: Tenant branding and workspace appearance gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Role and per-user permissions gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O79" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Business accent/background branding and light/dark workspace preferences keep each tenant recognizable without changing operational data.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Give staff only the workspaces and actions they need while business-level entitlements remain the ceiling.</x:v>
       </x:c>
       <x:c r="P79" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q79" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Tenant branding and workspace appearance. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Role and per-user permissions. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R79" s="13" t="str"/>
       <x:c r="S79" s="13" t="str">
-        <x:v>workspace-theming</x:v>
+        <x:v>roles</x:v>
       </x:c>
       <x:c r="T79" s="34" t="str"/>
       <x:c r="U79" s="13" t="str">
@@ -5937,7 +5967,7 @@
         <x:v>Week 12</x:v>
       </x:c>
       <x:c r="D80" s="13" t="str">
-        <x:v>governance</x:v>
+        <x:v>experience</x:v>
       </x:c>
       <x:c r="E80" s="13" t="str">
         <x:v>Control / verification</x:v>
@@ -5949,7 +5979,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H80" s="13" t="str">
-        <x:v>Founder-controlled subscription plans</x:v>
+        <x:v>Tenant branding and workspace appearance</x:v>
       </x:c>
       <x:c r="I80" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5964,23 +5994,23 @@
         <x:v>Instagram, LinkedIn</x:v>
       </x:c>
       <x:c r="M80" s="13" t="str">
-        <x:v>INPROFIC operators and plan-managed tenants</x:v>
+        <x:v>business owners and teams</x:v>
       </x:c>
       <x:c r="N80" s="13" t="str">
-        <x:v>Year-end control check: Founder-controlled subscription plans gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Tenant branding and workspace appearance gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O80" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Control plan pricing, module entitlements and commercial access without deleting tenant history.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Business accent/background branding and light/dark workspace preferences keep each tenant recognizable without changing operational data.</x:v>
       </x:c>
       <x:c r="P80" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q80" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Founder-controlled subscription plans. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Tenant branding and workspace appearance. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R80" s="13" t="str"/>
       <x:c r="S80" s="13" t="str">
-        <x:v>subscriptions</x:v>
+        <x:v>workspace-theming</x:v>
       </x:c>
       <x:c r="T80" s="34" t="str"/>
       <x:c r="U80" s="13" t="str">
@@ -6012,7 +6042,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H81" s="13" t="str">
-        <x:v>✨ NEW — Founder-controlled third-party integration availability</x:v>
+        <x:v>✨ NEW — Founder-controlled subscription plans &amp; trial policy</x:v>
       </x:c>
       <x:c r="I81" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -6027,28 +6057,28 @@
         <x:v>LinkedIn, Facebook</x:v>
       </x:c>
       <x:c r="M81" s="13" t="str">
-        <x:v>INPROFIC platform operators and businesses using optional delivery providers</x:v>
+        <x:v>INPROFIC operators and plan-managed tenants</x:v>
       </x:c>
       <x:c r="N81" s="13" t="str">
-        <x:v>Year-end control check: ✨ NEW — Founder-controlled third-party integration availability gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: ✨ NEW — Founder-controlled subscription plans &amp; trial policy gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O81" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Optional provider connectors can be hidden and execution-blocked platform-wide without deleting tenant credentials or history; businesses still activate their own approved provider accounts only after configuration.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Control plan pricing, module entitlements, the general free-trial duration and per-business founder trial extensions without deleting tenant history or overlapping active paid/lifetime access.</x:v>
       </x:c>
       <x:c r="P81" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q81" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Founder-controlled third-party integration availability. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Founder-controlled subscription plans &amp; trial policy. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R81" s="13" t="str">
         <x:v>NEW</x:v>
       </x:c>
       <x:c r="S81" s="13" t="str">
-        <x:v>founder-integration-gates</x:v>
+        <x:v>subscriptions</x:v>
       </x:c>
       <x:c r="T81" s="34" t="n">
-        <x:v>46285</x:v>
+        <x:v>46286</x:v>
       </x:c>
       <x:c r="U81" s="13" t="str">
         <x:v>Planned</x:v>
@@ -6079,7 +6109,7 @@
         <x:v>Consideration</x:v>
       </x:c>
       <x:c r="H82" s="13" t="str">
-        <x:v>Multiple service/business profiles under one subscription</x:v>
+        <x:v>✨ NEW — Founder-controlled third-party integration availability</x:v>
       </x:c>
       <x:c r="I82" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -6094,25 +6124,29 @@
         <x:v>Instagram, TikTok</x:v>
       </x:c>
       <x:c r="M82" s="13" t="str">
-        <x:v>owners running more than one service line</x:v>
+        <x:v>INPROFIC platform operators and businesses using optional delivery providers</x:v>
       </x:c>
       <x:c r="N82" s="13" t="str">
-        <x:v>Year-end control check: Multiple service/business profiles under one subscription gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: ✨ NEW — Founder-controlled third-party integration availability gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O82" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Provision additional tenant-isolated service profiles, carry appropriate memberships across, and switch between them without mixing records.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Optional provider connectors can be hidden and execution-blocked platform-wide without deleting tenant credentials or history; businesses still activate their own approved provider accounts only after configuration.</x:v>
       </x:c>
       <x:c r="P82" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q82" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Multiple service/business profiles under one subscription. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
-      </x:c>
-      <x:c r="R82" s="13" t="str"/>
+        <x:v>Use a real INPROFIC screen/demo for Founder-controlled third-party integration availability. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+      </x:c>
+      <x:c r="R82" s="13" t="str">
+        <x:v>NEW</x:v>
+      </x:c>
       <x:c r="S82" s="13" t="str">
-        <x:v>multi-service-profiles</x:v>
-      </x:c>
-      <x:c r="T82" s="34" t="str"/>
+        <x:v>founder-integration-gates</x:v>
+      </x:c>
+      <x:c r="T82" s="34" t="n">
+        <x:v>46285</x:v>
+      </x:c>
       <x:c r="U82" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -6142,7 +6176,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H83" s="13" t="str">
-        <x:v>✨ NEW — Plan-upgrade data continuity</x:v>
+        <x:v>Multiple service/business profiles under one subscription</x:v>
       </x:c>
       <x:c r="I83" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -6157,29 +6191,25 @@
         <x:v>Instagram Stories, Facebook Stories</x:v>
       </x:c>
       <x:c r="M83" s="13" t="str">
-        <x:v>owners evaluating plan upgrades</x:v>
+        <x:v>owners running more than one service line</x:v>
       </x:c>
       <x:c r="N83" s="13" t="str">
-        <x:v>Year-end control check: ✨ NEW — Plan-upgrade data continuity gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Multiple service/business profiles under one subscription gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O83" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Hidden interconnected modules do not stop required back-office synchronization, so upgrades reveal already-complete records.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Provision additional tenant-isolated service profiles, carry appropriate memberships across, and switch between them without mixing records.</x:v>
       </x:c>
       <x:c r="P83" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q83" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Plan-upgrade data continuity. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
-      </x:c>
-      <x:c r="R83" s="13" t="str">
-        <x:v>NEW</x:v>
-      </x:c>
+        <x:v>Use a real INPROFIC screen/demo for Multiple service/business profiles under one subscription. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+      </x:c>
+      <x:c r="R83" s="13" t="str"/>
       <x:c r="S83" s="13" t="str">
-        <x:v>entitlement-continuity</x:v>
-      </x:c>
-      <x:c r="T83" s="34" t="n">
-        <x:v>46285</x:v>
-      </x:c>
+        <x:v>multi-service-profiles</x:v>
+      </x:c>
+      <x:c r="T83" s="34" t="str"/>
       <x:c r="U83" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -6209,7 +6239,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H84" s="13" t="str">
-        <x:v>Reports, exports and business backup</x:v>
+        <x:v>✨ NEW — Plan-upgrade data continuity</x:v>
       </x:c>
       <x:c r="I84" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -6224,25 +6254,29 @@
         <x:v>LinkedIn, Facebook</x:v>
       </x:c>
       <x:c r="M84" s="13" t="str">
-        <x:v>owners, managers and auditors</x:v>
+        <x:v>owners evaluating plan upgrades</x:v>
       </x:c>
       <x:c r="N84" s="13" t="str">
-        <x:v>Year-end control check: Reports, exports and business backup gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: ✨ NEW — Plan-upgrade data continuity gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O84" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Export operational reports and maintain a tenant backup path without flattening audit history.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Hidden interconnected modules do not stop required back-office synchronization, so upgrades reveal already-complete records.</x:v>
       </x:c>
       <x:c r="P84" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q84" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Reports, exports and business backup. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
-      </x:c>
-      <x:c r="R84" s="13" t="str"/>
+        <x:v>Use a real INPROFIC screen/demo for Plan-upgrade data continuity. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+      </x:c>
+      <x:c r="R84" s="13" t="str">
+        <x:v>NEW</x:v>
+      </x:c>
       <x:c r="S84" s="13" t="str">
-        <x:v>reports-backup</x:v>
-      </x:c>
-      <x:c r="T84" s="34" t="str"/>
+        <x:v>entitlement-continuity</x:v>
+      </x:c>
+      <x:c r="T84" s="34" t="n">
+        <x:v>46285</x:v>
+      </x:c>
       <x:c r="U84" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -6260,7 +6294,7 @@
         <x:v>Week 12</x:v>
       </x:c>
       <x:c r="D85" s="13" t="str">
-        <x:v>experience</x:v>
+        <x:v>governance</x:v>
       </x:c>
       <x:c r="E85" s="13" t="str">
         <x:v>Screen / workflow demo</x:v>
@@ -6272,7 +6306,7 @@
         <x:v>Consideration</x:v>
       </x:c>
       <x:c r="H85" s="13" t="str">
-        <x:v>Guided system onboarding</x:v>
+        <x:v>Reports, exports and business backup</x:v>
       </x:c>
       <x:c r="I85" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -6287,23 +6321,23 @@
         <x:v>Instagram, Facebook, LinkedIn</x:v>
       </x:c>
       <x:c r="M85" s="13" t="str">
-        <x:v>new teams</x:v>
+        <x:v>owners, managers and auditors</x:v>
       </x:c>
       <x:c r="N85" s="13" t="str">
-        <x:v>Year-end control check: Guided system onboarding gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Reports, exports and business backup gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O85" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: A replayable module-aware tour helps staff learn the workspace without developer terminology.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Export operational reports and maintain a tenant backup path without flattening audit history.</x:v>
       </x:c>
       <x:c r="P85" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q85" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Guided system onboarding. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Reports, exports and business backup. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R85" s="13" t="str"/>
       <x:c r="S85" s="13" t="str">
-        <x:v>onboarding</x:v>
+        <x:v>reports-backup</x:v>
       </x:c>
       <x:c r="T85" s="34" t="str"/>
       <x:c r="U85" s="13" t="str">
@@ -6323,7 +6357,7 @@
         <x:v>Week 13</x:v>
       </x:c>
       <x:c r="D86" s="13" t="str">
-        <x:v>commerce</x:v>
+        <x:v>experience</x:v>
       </x:c>
       <x:c r="E86" s="13" t="str">
         <x:v>Connected-system handoff</x:v>
@@ -6335,7 +6369,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H86" s="13" t="str">
-        <x:v>✨ NEW — Surface-safe Online, POS and Distribution pricing</x:v>
+        <x:v>Guided system onboarding</x:v>
       </x:c>
       <x:c r="I86" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -6350,29 +6384,25 @@
         <x:v>Instagram, Facebook</x:v>
       </x:c>
       <x:c r="M86" s="13" t="str">
-        <x:v>businesses selling both in-premise and online</x:v>
+        <x:v>new teams</x:v>
       </x:c>
       <x:c r="N86" s="13" t="str">
-        <x:v>Year-end control check: ✨ NEW — Surface-safe Online, POS and Distribution pricing gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Guided system onboarding gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O86" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Physical Store/direct pricing stays inside the staff POS, while hosted/headless commerce exposes Online plus Distribution/Bulk and INPROFIC enforces the chosen channel and minimum quantity server-side.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: A replayable tenant-aware tour keeps the original animated guide and adds a second module-specific preview that reflects the business vertical.</x:v>
       </x:c>
       <x:c r="P86" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q86" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Surface-safe Online, POS and Distribution pricing. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
-      </x:c>
-      <x:c r="R86" s="13" t="str">
-        <x:v>NEW</x:v>
-      </x:c>
+        <x:v>Use a real INPROFIC screen/demo for Guided system onboarding. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+      </x:c>
+      <x:c r="R86" s="13" t="str"/>
       <x:c r="S86" s="13" t="str">
-        <x:v>commerce-channel-boundary</x:v>
-      </x:c>
-      <x:c r="T86" s="34" t="n">
-        <x:v>46285</x:v>
-      </x:c>
+        <x:v>onboarding</x:v>
+      </x:c>
+      <x:c r="T86" s="34" t="str"/>
       <x:c r="U86" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -6402,7 +6432,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H87" s="13" t="str">
-        <x:v>✨ NEW — Standard portions, composed products and Bulk Packs</x:v>
+        <x:v>✨ NEW — Surface-safe Online, POS and Distribution pricing</x:v>
       </x:c>
       <x:c r="I87" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -6417,25 +6447,25 @@
         <x:v>Instagram, LinkedIn</x:v>
       </x:c>
       <x:c r="M87" s="13" t="str">
-        <x:v>restaurants and production businesses selling in customer-friendly portions or bulk packs</x:v>
+        <x:v>businesses selling both in-premise and online</x:v>
       </x:c>
       <x:c r="N87" s="13" t="str">
-        <x:v>Year-end control check: ✨ NEW — Standard portions, composed products and Bulk Packs gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: ✨ NEW — Surface-safe Online, POS and Distribution pricing gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O87" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Keep production in base units such as scoops/pieces/ml while customers buy plates, servings, bowls, cartons or other packs; show customer-safe package contents and preserve private yield conversions.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Physical Store/direct pricing stays inside the staff POS, while hosted/headless commerce exposes Online plus Distribution/Bulk and INPROFIC enforces the chosen channel and minimum quantity server-side.</x:v>
       </x:c>
       <x:c r="P87" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q87" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Standard portions, composed products and Bulk Packs. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Surface-safe Online, POS and Distribution pricing. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R87" s="13" t="str">
         <x:v>NEW</x:v>
       </x:c>
       <x:c r="S87" s="13" t="str">
-        <x:v>portion-bulk-pack-composition</x:v>
+        <x:v>commerce-channel-boundary</x:v>
       </x:c>
       <x:c r="T87" s="34" t="n">
         <x:v>46285</x:v>
@@ -6457,7 +6487,7 @@
         <x:v>Week 13</x:v>
       </x:c>
       <x:c r="D88" s="13" t="str">
-        <x:v>governance</x:v>
+        <x:v>commerce</x:v>
       </x:c>
       <x:c r="E88" s="13" t="str">
         <x:v>Persona / use case</x:v>
@@ -6469,7 +6499,7 @@
         <x:v>Consideration</x:v>
       </x:c>
       <x:c r="H88" s="13" t="str">
-        <x:v>✨ NEW — Founder product and lead analytics</x:v>
+        <x:v>✨ NEW — Standard portions, composed products and Bulk Packs</x:v>
       </x:c>
       <x:c r="I88" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -6484,25 +6514,25 @@
         <x:v>LinkedIn, Facebook</x:v>
       </x:c>
       <x:c r="M88" s="13" t="str">
-        <x:v>INPROFIC founders and platform operators</x:v>
+        <x:v>restaurants and production businesses selling in customer-friendly portions or bulk packs</x:v>
       </x:c>
       <x:c r="N88" s="13" t="str">
-        <x:v>Year-end control check: ✨ NEW — Founder product and lead analytics gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: ✨ NEW — Standard portions, composed products and Bulk Packs gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O88" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Track first-party signup leads, completed registrations, logins, subscription milestones and throttled module usage in Founder Console without recording passwords, payment secrets or arbitrary clickstreams.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Keep production in base units such as scoops/pieces/ml while customers buy plates, servings, bowls, cartons or other packs; show customer-safe package contents and preserve private yield conversions.</x:v>
       </x:c>
       <x:c r="P88" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q88" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Founder product and lead analytics. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Standard portions, composed products and Bulk Packs. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R88" s="13" t="str">
         <x:v>NEW</x:v>
       </x:c>
       <x:c r="S88" s="13" t="str">
-        <x:v>founder-product-analytics</x:v>
+        <x:v>portion-bulk-pack-composition</x:v>
       </x:c>
       <x:c r="T88" s="34" t="n">
         <x:v>46285</x:v>
@@ -6524,7 +6554,7 @@
         <x:v>Week 13</x:v>
       </x:c>
       <x:c r="D89" s="13" t="str">
-        <x:v>experience</x:v>
+        <x:v>governance</x:v>
       </x:c>
       <x:c r="E89" s="13" t="str">
         <x:v>Recap / CTA</x:v>
@@ -6536,7 +6566,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H89" s="13" t="str">
-        <x:v>✨ NEW — Animated, consistent form validation across INPROFIC</x:v>
+        <x:v>✨ NEW — Founder product and lead analytics</x:v>
       </x:c>
       <x:c r="I89" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -6551,25 +6581,25 @@
         <x:v>Instagram, TikTok</x:v>
       </x:c>
       <x:c r="M89" s="13" t="str">
-        <x:v>staff and hosted-storefront customers</x:v>
+        <x:v>INPROFIC founders and platform operators</x:v>
       </x:c>
       <x:c r="N89" s="13" t="str">
-        <x:v>Year-end control check: ✨ NEW — Animated, consistent form validation across INPROFIC gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: ✨ NEW — Founder product and lead analytics gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O89" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: HTML5 and Django validation share animated field states, contextual SVG affordances, accessible feedback and consistent toggle switches; dynamic rows inherit the same behavior.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Track first-party signup leads, completed registrations, logins, subscription milestones and throttled module usage in Founder Console without recording passwords, payment secrets or arbitrary clickstreams.</x:v>
       </x:c>
       <x:c r="P89" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q89" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Animated, consistent form validation across INPROFIC. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Founder product and lead analytics. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R89" s="13" t="str">
         <x:v>NEW</x:v>
       </x:c>
       <x:c r="S89" s="13" t="str">
-        <x:v>form-experience-v2</x:v>
+        <x:v>founder-product-analytics</x:v>
       </x:c>
       <x:c r="T89" s="34" t="n">
         <x:v>46285</x:v>
@@ -6591,7 +6621,7 @@
         <x:v>Week 13</x:v>
       </x:c>
       <x:c r="D90" s="13" t="str">
-        <x:v>commerce</x:v>
+        <x:v>experience</x:v>
       </x:c>
       <x:c r="E90" s="13" t="str">
         <x:v>Problem / pain point</x:v>
@@ -6603,7 +6633,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H90" s="13" t="str">
-        <x:v>✨ NEW — Channel-aware plain and add-on product options</x:v>
+        <x:v>✨ NEW — Animated, consistent form validation across INPROFIC</x:v>
       </x:c>
       <x:c r="I90" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -6618,25 +6648,25 @@
         <x:v>Instagram Stories, Facebook Stories</x:v>
       </x:c>
       <x:c r="M90" s="13" t="str">
-        <x:v>restaurants and production businesses selling composed products plus extras</x:v>
+        <x:v>staff and hosted-storefront customers</x:v>
       </x:c>
       <x:c r="N90" s="13" t="str">
-        <x:v>Year-end control check: ✨ NEW — Channel-aware plain and add-on product options gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: ✨ NEW — Animated, consistent form validation across INPROFIC gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O90" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Offer Extra Jollof, Single Chicken, bottles, pieces or other plain portions from the same Finished Good stock and recipe with independent Physical Store, Online and Bulk/Distribution availability and pricing.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: HTML5 and Django validation share animated field states, contextual SVG affordances, accessible feedback and consistent toggle switches; dynamic rows inherit the same behavior.</x:v>
       </x:c>
       <x:c r="P90" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q90" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Channel-aware plain and add-on product options. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Animated, consistent form validation across INPROFIC. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R90" s="13" t="str">
         <x:v>NEW</x:v>
       </x:c>
       <x:c r="S90" s="13" t="str">
-        <x:v>individual-sale-options</x:v>
+        <x:v>form-experience-v2</x:v>
       </x:c>
       <x:c r="T90" s="34" t="n">
         <x:v>46285</x:v>
@@ -6658,7 +6688,7 @@
         <x:v>Week 13</x:v>
       </x:c>
       <x:c r="D91" s="13" t="str">
-        <x:v>operations</x:v>
+        <x:v>commerce</x:v>
       </x:c>
       <x:c r="E91" s="13" t="str">
         <x:v>How it works</x:v>
@@ -6670,7 +6700,7 @@
         <x:v>Consideration</x:v>
       </x:c>
       <x:c r="H91" s="13" t="str">
-        <x:v>Inventory with purchase-to-usage units</x:v>
+        <x:v>✨ NEW — Channel-aware plain and add-on product options</x:v>
       </x:c>
       <x:c r="I91" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -6685,25 +6715,29 @@
         <x:v>LinkedIn, Facebook</x:v>
       </x:c>
       <x:c r="M91" s="13" t="str">
-        <x:v>owners, storekeepers, production teams</x:v>
+        <x:v>restaurants and production businesses selling composed products plus extras</x:v>
       </x:c>
       <x:c r="N91" s="13" t="str">
-        <x:v>Year-end control check: Inventory with purchase-to-usage units gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: ✨ NEW — Channel-aware plain and add-on product options gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O91" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Buy in packs or bags while stock and recipes stay accurate in the unit actually consumed.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Offer Extra Jollof, Single Chicken, bottles, pieces or other plain portions from the same Finished Good stock and recipe with independent Physical Store, Online and Bulk/Distribution availability and pricing.</x:v>
       </x:c>
       <x:c r="P91" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q91" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Inventory with purchase-to-usage units. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
-      </x:c>
-      <x:c r="R91" s="13" t="str"/>
+        <x:v>Use a real INPROFIC screen/demo for Channel-aware plain and add-on product options. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+      </x:c>
+      <x:c r="R91" s="13" t="str">
+        <x:v>NEW</x:v>
+      </x:c>
       <x:c r="S91" s="13" t="str">
-        <x:v>inventory-units</x:v>
-      </x:c>
-      <x:c r="T91" s="34" t="str"/>
+        <x:v>individual-sale-options</x:v>
+      </x:c>
+      <x:c r="T91" s="34" t="n">
+        <x:v>46285</x:v>
+      </x:c>
       <x:c r="U91" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -6733,7 +6767,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H92" s="13" t="str">
-        <x:v>Dashboard search and operating insights</x:v>
+        <x:v>✨ NEW — Interactive product demos</x:v>
       </x:c>
       <x:c r="I92" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -6748,25 +6782,29 @@
         <x:v>Instagram, Facebook, LinkedIn</x:v>
       </x:c>
       <x:c r="M92" s="13" t="str">
-        <x:v>owners and managers</x:v>
+        <x:v>prospective businesses exploring INPROFIC</x:v>
       </x:c>
       <x:c r="N92" s="13" t="str">
-        <x:v>Year-end control check: Dashboard search and operating insights gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: ✨ NEW — Interactive product demos gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O92" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Search key business records quickly and review stock, commercial and period signals from one operating dashboard.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: The marketing site provides a vertical-aware click-through workflow plus module-card flip previews and a detailed storefront-to-fulfilment flow.</x:v>
       </x:c>
       <x:c r="P92" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q92" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Dashboard search and operating insights. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
-      </x:c>
-      <x:c r="R92" s="13" t="str"/>
+        <x:v>Use a real INPROFIC screen/demo for Interactive product demos. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+      </x:c>
+      <x:c r="R92" s="13" t="str">
+        <x:v>NEW</x:v>
+      </x:c>
       <x:c r="S92" s="13" t="str">
-        <x:v>dashboard-insights</x:v>
-      </x:c>
-      <x:c r="T92" s="34" t="str"/>
+        <x:v>interactive-product-demos</x:v>
+      </x:c>
+      <x:c r="T92" s="34" t="n">
+        <x:v>46286</x:v>
+      </x:c>
       <x:c r="U92" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -6796,7 +6834,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H93" s="13" t="str">
-        <x:v>✨ NEW — Persistent stock alerts inside the shared operations tray</x:v>
+        <x:v>Inventory with purchase-to-usage units</x:v>
       </x:c>
       <x:c r="I93" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -6811,29 +6849,25 @@
         <x:v>Instagram, Facebook</x:v>
       </x:c>
       <x:c r="M93" s="13" t="str">
-        <x:v>owners, storekeepers, managers</x:v>
+        <x:v>owners, storekeepers, production teams</x:v>
       </x:c>
       <x:c r="N93" s="13" t="str">
-        <x:v>Year-end control check: ✨ NEW — Persistent stock alerts inside the shared operations tray gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: Inventory with purchase-to-usage units gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O93" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Raw-material and finished-good warning/low conditions open in separate Inventory tabs inside the movable tray, keep per-user snooze/re-alert timing, repeat a chosen INPROFIC tune in the foreground, and continue due reminders through Web Push when the app is backgrounded or closed.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Buy in packs or bags while stock and recipes stay accurate in the unit actually consumed.</x:v>
       </x:c>
       <x:c r="P93" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q93" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Persistent stock alerts inside the shared operations tray. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
-      </x:c>
-      <x:c r="R93" s="13" t="str">
-        <x:v>NEW</x:v>
-      </x:c>
+        <x:v>Use a real INPROFIC screen/demo for Inventory with purchase-to-usage units. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+      </x:c>
+      <x:c r="R93" s="13" t="str"/>
       <x:c r="S93" s="13" t="str">
-        <x:v>stock-alerts</x:v>
-      </x:c>
-      <x:c r="T93" s="34" t="n">
-        <x:v>46285</x:v>
-      </x:c>
+        <x:v>inventory-units</x:v>
+      </x:c>
+      <x:c r="T93" s="34" t="str"/>
       <x:c r="U93" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -6861,7 +6895,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R382b744514df47e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd068d161c98a4a15"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6954,7 +6988,7 @@
         <x:v>owners, storekeepers, managers</x:v>
       </x:c>
       <x:c r="E4" s="13" t="str">
-        <x:v>Raw-material and finished-good warning/low conditions open in separate Inventory tabs inside the movable tray, keep per-user snooze/re-alert timing, repeat a chosen INPROFIC tune in the foreground, and continue due reminders through Web Push when the app is backgrounded or closed.</x:v>
+        <x:v>Raw-material and finished-good warning/low conditions open in separate Inventory tabs inside the movable tray, keep per-user snooze/re-alert timing, can use synthesized alerts or eight bundled audio chimes, and continue due reminders through Web Push when the app is backgrounded or closed.</x:v>
       </x:c>
       <x:c r="F4" s="13" t="str">
         <x:v>NEW</x:v>
@@ -7034,7 +7068,7 @@
         <x:v>wholesalers and retailers</x:v>
       </x:c>
       <x:c r="E8" s="13" t="str">
-        <x:v>Procure and sell resale products without forcing them through Production.</x:v>
+        <x:v>Wholesale and retail use procurement-first stock-product forms and supporting-supply controls without production-only recipe, batch or base-material fields.</x:v>
       </x:c>
       <x:c r="F8" s="13" t="str"/>
       <x:c r="G8" s="34"/>
@@ -7384,7 +7418,7 @@
         <x:v>dispatchers, managers and riders</x:v>
       </x:c>
       <x:c r="E26" s="13" t="str">
-        <x:v>Commerce, payment and Delivery alerts share one movable tray with Inventory without sharing read state; five selectable foreground tunes and configurable repeats keep unread work—including direct Transfer verification—hard to miss, while durable Web Push continues due reminders in the background.</x:v>
+        <x:v>Commerce, payment and Delivery alerts share one movable tray with Inventory without sharing read state; synthesized tones plus eight bundled audio chimes and configurable repeats keep unread work—including direct Transfer verification—hard to miss, while durable Web Push continues due reminders in the background.</x:v>
       </x:c>
       <x:c r="F26" s="13" t="str">
         <x:v>NEW</x:v>
@@ -7493,7 +7527,7 @@
         <x:v>subscriptions</x:v>
       </x:c>
       <x:c r="B32" s="13" t="str">
-        <x:v>Founder-controlled subscription plans</x:v>
+        <x:v>Founder-controlled subscription plans &amp; trial policy</x:v>
       </x:c>
       <x:c r="C32" s="13" t="str">
         <x:v>governance</x:v>
@@ -7502,10 +7536,14 @@
         <x:v>INPROFIC operators and plan-managed tenants</x:v>
       </x:c>
       <x:c r="E32" s="13" t="str">
-        <x:v>Control plan pricing, module entitlements and commercial access without deleting tenant history.</x:v>
-      </x:c>
-      <x:c r="F32" s="13" t="str"/>
-      <x:c r="G32" s="34"/>
+        <x:v>Control plan pricing, module entitlements, the general free-trial duration and per-business founder trial extensions without deleting tenant history or overlapping active paid/lifetime access.</x:v>
+      </x:c>
+      <x:c r="F32" s="13" t="str">
+        <x:v>NEW</x:v>
+      </x:c>
+      <x:c r="G32" s="34" t="n">
+        <x:v>46286</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="13" t="str">
@@ -7605,7 +7643,7 @@
         <x:v>new teams</x:v>
       </x:c>
       <x:c r="E37" s="13" t="str">
-        <x:v>A replayable module-aware tour helps staff learn the workspace without developer terminology.</x:v>
+        <x:v>A replayable tenant-aware tour keeps the original animated guide and adds a second module-specific preview that reflects the business vertical.</x:v>
       </x:c>
       <x:c r="F37" s="13" t="str"/>
       <x:c r="G37" s="34"/>
@@ -7725,15 +7763,38 @@
         <x:v>46285</x:v>
       </x:c>
     </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="13" t="str">
+        <x:v>interactive-product-demos</x:v>
+      </x:c>
+      <x:c r="B43" s="13" t="str">
+        <x:v>Interactive product demos</x:v>
+      </x:c>
+      <x:c r="C43" s="13" t="str">
+        <x:v>experience</x:v>
+      </x:c>
+      <x:c r="D43" s="13" t="str">
+        <x:v>prospective businesses exploring INPROFIC</x:v>
+      </x:c>
+      <x:c r="E43" s="13" t="str">
+        <x:v>The marketing site provides a vertical-aware click-through workflow plus module-card flip previews and a detailed storefront-to-fulfilment flow.</x:v>
+      </x:c>
+      <x:c r="F43" s="13" t="str">
+        <x:v>NEW</x:v>
+      </x:c>
+      <x:c r="G43" s="34" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="F2:F42">
+  <x:conditionalFormatting sqref="F2:F43">
     <x:cfRule type="expression" dxfId="3" priority="1">
       <x:formula>F2="NEW"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde1f8166bbf64930"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c3e60c40e3e4727"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Onboarding Tour Bug Fix
</commit_message>
<xml_diff>
--- a/docs/INPROFIC_Q4_2026_Content_Calendar.xlsx
+++ b/docs/INPROFIC_Q4_2026_Content_Calendar.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Summary" sheetId="1" r:id="Rd516e238f33f4c9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendar" sheetId="2" r:id="R51b74aa8e87c4e32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Catalog" sheetId="3" r:id="R262b37945c0e4d55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Guide" sheetId="4" r:id="Raca407a3e62a46a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Summary" sheetId="1" r:id="R4824374e891f4adf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendar" sheetId="2" r:id="R2499b046a6ec4b36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Catalog" sheetId="3" r:id="R5cc3f64539314e88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Guide" sheetId="4" r:id="R155973ebddbb46e0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -601,7 +601,7 @@
       </x:c>
       <x:c r="B6" t="n">
         <x:f>COUNTIF('Feature Catalog'!F2:F200,"NEW")</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D6" s="13" t="str">
         <x:v>November</x:v>
@@ -711,21 +711,21 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="32" t="str">
-        <x:v>Provider-neutral delivery partner adapters</x:v>
+        <x:v>In-premise POS</x:v>
       </x:c>
       <x:c r="B16" s="13" t="str">
-        <x:v>Keep INPROFIC in control of delivery pricing, routing and tracking while any courier stays manual or connects through a normalized dispatch/status adapter; optional built-in providers remain separately governed.</x:v>
+        <x:v>Staff can complete counter sales with Cash, direct Transfer or supported terminal payment only when the tenant plan includes Commerce and Commerce is explicitly enabled; POS still keeps its dedicated user permission.</x:v>
       </x:c>
       <x:c r="C16" s="34" t="n">
-        <x:v>46285</x:v>
+        <x:v>46289</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="32" t="str">
-        <x:v>Shared realtime Commerce, payment and delivery alert tray</x:v>
+        <x:v>Provider-neutral delivery partner adapters</x:v>
       </x:c>
       <x:c r="B17" s="13" t="str">
-        <x:v>Commerce, payment and Delivery alerts share one movable tray with Inventory without sharing read state; synthesized tones plus eight bundled audio chimes and configurable repeats keep unread work—including direct Transfer verification—hard to miss, while durable Web Push continues due reminders in the background.</x:v>
+        <x:v>Keep INPROFIC in control of delivery pricing, routing and tracking while any courier stays manual or connects through a normalized dispatch/status adapter; optional built-in providers remain separately governed.</x:v>
       </x:c>
       <x:c r="C17" s="34" t="n">
         <x:v>46285</x:v>
@@ -733,24 +733,24 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="32" t="str">
-        <x:v>Founder-controlled subscription plans &amp; trial policy</x:v>
+        <x:v>Shared realtime Commerce, Inventory and Finance alert tray</x:v>
       </x:c>
       <x:c r="B18" s="13" t="str">
-        <x:v>Control plan pricing, module entitlements, the general free-trial duration and per-business founder trial extensions without deleting tenant history or overlapping active paid/lifetime access.</x:v>
+        <x:v>Commerce, payment, Delivery, Inventory and Finance attention share one movable access-aware tray without merging their underlying record state; Commerce/Delivery can use durable Web Push in the background, while Finance surfaces unpaid invoices, receivables, payables and balancing anomalies from the same finance records.</x:v>
       </x:c>
       <x:c r="C18" s="34" t="n">
-        <x:v>46286</x:v>
+        <x:v>46289</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="32" t="str">
-        <x:v>Founder-controlled third-party integration availability</x:v>
+        <x:v>Founder-controlled subscription plans &amp; trial policy</x:v>
       </x:c>
       <x:c r="B19" s="13" t="str">
-        <x:v>Optional provider connectors can be hidden and execution-blocked platform-wide without deleting tenant credentials or history; businesses still activate their own approved provider accounts only after configuration.</x:v>
+        <x:v>Control plan pricing, module entitlements, the general free-trial duration and per-business founder trial extensions without deleting tenant history or overlapping active paid/lifetime access.</x:v>
       </x:c>
       <x:c r="C19" s="34" t="n">
-        <x:v>46285</x:v>
+        <x:v>46286</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
@@ -758,7 +758,7 @@
         <x:v>Maintenance rule: whenever a user-visible INPROFIC capability is added or materially changed, update docs/feature_marketing_catalog.json and run scripts/generate_marketing_calendar.py. The CSV, Markdown and Excel outputs are regenerated together; new additions remain visibly marked ✨ NEW.</x:v>
       </x:c>
       <x:c r="B20" s="41" t="str">
-        <x:v>Hidden interconnected modules do not stop required back-office synchronization, so upgrades reveal already-complete records.</x:v>
+        <x:v>Optional provider connectors can be hidden and execution-blocked platform-wide without deleting tenant credentials or history; businesses still activate their own approved provider accounts only after configuration.</x:v>
       </x:c>
       <x:c r="C20" s="42" t="n">
         <x:v>46285</x:v>
@@ -771,10 +771,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32" t="str">
-        <x:v>Surface-safe Online, POS and Distribution pricing</x:v>
+        <x:v>Plan-upgrade data continuity</x:v>
       </x:c>
       <x:c r="B21" s="13" t="str">
-        <x:v>Physical Store/direct pricing stays inside the staff POS, while hosted/headless commerce exposes Online plus Distribution/Bulk and INPROFIC enforces the chosen channel and minimum quantity server-side.</x:v>
+        <x:v>Hidden interconnected modules do not stop required back-office synchronization, so upgrades reveal already-complete records.</x:v>
       </x:c>
       <x:c r="C21" s="34" t="n">
         <x:v>46285</x:v>
@@ -782,10 +782,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="32" t="str">
-        <x:v>Standard portions, composed products and Bulk Packs</x:v>
+        <x:v>Surface-safe Online, POS and Distribution pricing</x:v>
       </x:c>
       <x:c r="B22" s="13" t="str">
-        <x:v>Keep production in base units such as scoops/pieces/ml while customers buy plates, servings, bowls, cartons or other packs; show customer-safe package contents and preserve private yield conversions.</x:v>
+        <x:v>Physical Store/direct pricing stays inside the staff POS, while hosted/headless commerce exposes Online plus Distribution/Bulk and INPROFIC enforces the chosen channel and minimum quantity server-side.</x:v>
       </x:c>
       <x:c r="C22" s="34" t="n">
         <x:v>46285</x:v>
@@ -793,10 +793,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="32" t="str">
-        <x:v>Founder product and lead analytics</x:v>
+        <x:v>Standard portions, composed products and Bulk Packs</x:v>
       </x:c>
       <x:c r="B23" s="13" t="str">
-        <x:v>Track first-party signup leads, completed registrations, logins, subscription milestones and throttled module usage in Founder Console without recording passwords, payment secrets or arbitrary clickstreams.</x:v>
+        <x:v>Keep production in base units such as scoops/pieces/ml while customers buy plates, servings, bowls, cartons or other packs; show customer-safe package contents and preserve private yield conversions.</x:v>
       </x:c>
       <x:c r="C23" s="34" t="n">
         <x:v>46285</x:v>
@@ -804,21 +804,21 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32" t="str">
-        <x:v>Animated, consistent form validation across INPROFIC</x:v>
+        <x:v>Founder product and lead analytics</x:v>
       </x:c>
       <x:c r="B24" s="13" t="str">
-        <x:v>HTML5 and Django validation share animated field states, contextual SVG affordances, accessible feedback and consistent toggle switches; dynamic rows inherit the same behavior.</x:v>
+        <x:v>Track first-party signup leads, completed registrations, logins, subscription milestones and throttled module usage in Founder Console, with retained deleted-state and permanent-removal controls for signup mailing-list entries, without recording passwords, payment secrets or arbitrary clickstreams.</x:v>
       </x:c>
       <x:c r="C24" s="34" t="n">
-        <x:v>46285</x:v>
+        <x:v>46289</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32" t="str">
-        <x:v>Channel-aware plain and add-on product options</x:v>
+        <x:v>Animated, consistent form validation across INPROFIC</x:v>
       </x:c>
       <x:c r="B25" s="13" t="str">
-        <x:v>Offer Extra Jollof, Single Chicken, bottles, pieces or other plain portions from the same Finished Good stock and recipe with independent Physical Store, Online and Bulk/Distribution availability and pricing.</x:v>
+        <x:v>HTML5 and Django validation share animated field states, contextual SVG affordances, accessible feedback and consistent toggle switches; dynamic rows inherit the same behavior.</x:v>
       </x:c>
       <x:c r="C25" s="34" t="n">
         <x:v>46285</x:v>
@@ -826,12 +826,23 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32" t="str">
+        <x:v>Channel-aware plain and add-on product options</x:v>
+      </x:c>
+      <x:c r="B26" s="13" t="str">
+        <x:v>Offer Extra Jollof, Single Chicken, bottles, pieces or other plain portions from the same Finished Good stock and recipe with independent Physical Store, Online and Bulk/Distribution availability and pricing.</x:v>
+      </x:c>
+      <x:c r="C26" s="34" t="n">
+        <x:v>46285</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="32" t="str">
         <x:v>Interactive product demos</x:v>
       </x:c>
-      <x:c r="B26" s="13" t="str">
+      <x:c r="B27" s="13" t="str">
         <x:v>The marketing site provides a vertical-aware click-through workflow plus module-card flip previews and a detailed storefront-to-fulfilment flow.</x:v>
       </x:c>
-      <x:c r="C26" s="34" t="n">
+      <x:c r="C27" s="34" t="n">
         <x:v>46286</x:v>
       </x:c>
     </x:row>
@@ -2706,7 +2717,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H29" s="13" t="str">
-        <x:v>In-premise POS</x:v>
+        <x:v>✨ NEW — In-premise POS</x:v>
       </x:c>
       <x:c r="I29" s="13" t="str">
         <x:v>Feature education</x:v>
@@ -2724,10 +2735,10 @@
         <x:v>cashiers, stores, restaurants and walk-in operations</x:v>
       </x:c>
       <x:c r="N29" s="13" t="str">
-        <x:v>In-premise POS: what changes when this is handled inside one connected system?</x:v>
+        <x:v>✨ NEW — In-premise POS: what changes when this is handled inside one connected system?</x:v>
       </x:c>
       <x:c r="O29" s="13" t="str">
-        <x:v>Show exactly what the feature does and the workflow it replaces. Proof point: Staff can complete counter sales with Cash, direct Transfer or supported terminal payment without opening the wider workspace.</x:v>
+        <x:v>Show exactly what the feature does and the workflow it replaces. Proof point: Staff can complete counter sales with Cash, direct Transfer or supported terminal payment only when the tenant plan includes Commerce and Commerce is explicitly enabled; POS still keeps its dedicated user permission.</x:v>
       </x:c>
       <x:c r="P29" s="13" t="str">
         <x:v>See how it works</x:v>
@@ -2735,11 +2746,15 @@
       <x:c r="Q29" s="13" t="str">
         <x:v>Use a real INPROFIC screen/demo for In-premise POS. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
-      <x:c r="R29" s="13" t="str"/>
+      <x:c r="R29" s="13" t="str">
+        <x:v>NEW</x:v>
+      </x:c>
       <x:c r="S29" s="13" t="str">
         <x:v>pos</x:v>
       </x:c>
-      <x:c r="T29" s="34" t="str"/>
+      <x:c r="T29" s="34" t="n">
+        <x:v>46289</x:v>
+      </x:c>
       <x:c r="U29" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -2962,7 +2977,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H33" s="13" t="str">
-        <x:v>✨ NEW — Shared realtime Commerce, payment and delivery alert tray</x:v>
+        <x:v>✨ NEW — Shared realtime Commerce, Inventory and Finance alert tray</x:v>
       </x:c>
       <x:c r="I33" s="13" t="str">
         <x:v>Problem → workflow</x:v>
@@ -2980,16 +2995,16 @@
         <x:v>dispatchers, managers and riders</x:v>
       </x:c>
       <x:c r="N33" s="13" t="str">
-        <x:v>Still solving this manually? ✨ NEW — Shared realtime Commerce, payment and delivery alert tray keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
+        <x:v>Still solving this manually? ✨ NEW — Shared realtime Commerce, Inventory and Finance alert tray keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O33" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Commerce, payment and Delivery alerts share one movable tray with Inventory without sharing read state; synthesized tones plus eight bundled audio chimes and configurable repeats keep unread work—including direct Transfer verification—hard to miss, while durable Web Push continues due reminders in the background.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Commerce, payment, Delivery, Inventory and Finance attention share one movable access-aware tray without merging their underlying record state; Commerce/Delivery can use durable Web Push in the background, while Finance surfaces unpaid invoices, receivables, payables and balancing anomalies from the same finance records.</x:v>
       </x:c>
       <x:c r="P33" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
       </x:c>
       <x:c r="Q33" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Shared realtime Commerce, payment and delivery alert tray. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Shared realtime Commerce, Inventory and Finance alert tray. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R33" s="13" t="str">
         <x:v>NEW</x:v>
@@ -2998,7 +3013,7 @@
         <x:v>delivery-notifications</x:v>
       </x:c>
       <x:c r="T33" s="34" t="n">
-        <x:v>46285</x:v>
+        <x:v>46289</x:v>
       </x:c>
       <x:c r="U33" s="13" t="str">
         <x:v>Planned</x:v>
@@ -3889,7 +3904,7 @@
         <x:v>Still solving this manually? ✨ NEW — Founder product and lead analytics keeps the workflow connected instead of handing it off to another spreadsheet.</x:v>
       </x:c>
       <x:c r="O47" s="13" t="str">
-        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Track first-party signup leads, completed registrations, logins, subscription milestones and throttled module usage in Founder Console without recording passwords, payment secrets or arbitrary clickstreams.</x:v>
+        <x:v>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Track first-party signup leads, completed registrations, logins, subscription milestones and throttled module usage in Founder Console, with retained deleted-state and permanent-removal controls for signup mailing-list entries, without recording passwords, payment secrets or arbitrary clickstreams.</x:v>
       </x:c>
       <x:c r="P47" s="13" t="str">
         <x:v>Map this to your workflow</x:v>
@@ -3904,7 +3919,7 @@
         <x:v>founder-product-analytics</x:v>
       </x:c>
       <x:c r="T47" s="34" t="n">
-        <x:v>46285</x:v>
+        <x:v>46289</x:v>
       </x:c>
       <x:c r="U47" s="13" t="str">
         <x:v>Planned</x:v>
@@ -5404,7 +5419,7 @@
         <x:v>Conversion support</x:v>
       </x:c>
       <x:c r="H71" s="13" t="str">
-        <x:v>In-premise POS</x:v>
+        <x:v>✨ NEW — In-premise POS</x:v>
       </x:c>
       <x:c r="I71" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5422,10 +5437,10 @@
         <x:v>cashiers, stores, restaurants and walk-in operations</x:v>
       </x:c>
       <x:c r="N71" s="13" t="str">
-        <x:v>Year-end control check: In-premise POS gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: ✨ NEW — In-premise POS gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O71" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Staff can complete counter sales with Cash, direct Transfer or supported terminal payment without opening the wider workspace.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Staff can complete counter sales with Cash, direct Transfer or supported terminal payment only when the tenant plan includes Commerce and Commerce is explicitly enabled; POS still keeps its dedicated user permission.</x:v>
       </x:c>
       <x:c r="P71" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
@@ -5433,11 +5448,15 @@
       <x:c r="Q71" s="13" t="str">
         <x:v>Use a real INPROFIC screen/demo for In-premise POS. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
-      <x:c r="R71" s="13" t="str"/>
+      <x:c r="R71" s="13" t="str">
+        <x:v>NEW</x:v>
+      </x:c>
       <x:c r="S71" s="13" t="str">
         <x:v>pos</x:v>
       </x:c>
-      <x:c r="T71" s="34" t="str"/>
+      <x:c r="T71" s="34" t="n">
+        <x:v>46289</x:v>
+      </x:c>
       <x:c r="U71" s="13" t="str">
         <x:v>Planned</x:v>
       </x:c>
@@ -5660,7 +5679,7 @@
         <x:v>Awareness</x:v>
       </x:c>
       <x:c r="H75" s="13" t="str">
-        <x:v>✨ NEW — Shared realtime Commerce, payment and delivery alert tray</x:v>
+        <x:v>✨ NEW — Shared realtime Commerce, Inventory and Finance alert tray</x:v>
       </x:c>
       <x:c r="I75" s="13" t="str">
         <x:v>Control / ROI / readiness</x:v>
@@ -5678,16 +5697,16 @@
         <x:v>dispatchers, managers and riders</x:v>
       </x:c>
       <x:c r="N75" s="13" t="str">
-        <x:v>Year-end control check: ✨ NEW — Shared realtime Commerce, payment and delivery alert tray gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
+        <x:v>Year-end control check: ✨ NEW — Shared realtime Commerce, Inventory and Finance alert tray gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O75" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Commerce, payment and Delivery alerts share one movable tray with Inventory without sharing read state; synthesized tones plus eight bundled audio chimes and configurable repeats keep unread work—including direct Transfer verification—hard to miss, while durable Web Push continues due reminders in the background.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Commerce, payment, Delivery, Inventory and Finance attention share one movable access-aware tray without merging their underlying record state; Commerce/Delivery can use durable Web Push in the background, while Finance surfaces unpaid invoices, receivables, payables and balancing anomalies from the same finance records.</x:v>
       </x:c>
       <x:c r="P75" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
       </x:c>
       <x:c r="Q75" s="13" t="str">
-        <x:v>Use a real INPROFIC screen/demo for Shared realtime Commerce, payment and delivery alert tray. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
+        <x:v>Use a real INPROFIC screen/demo for Shared realtime Commerce, Inventory and Finance alert tray. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</x:v>
       </x:c>
       <x:c r="R75" s="13" t="str">
         <x:v>NEW</x:v>
@@ -5696,7 +5715,7 @@
         <x:v>delivery-notifications</x:v>
       </x:c>
       <x:c r="T75" s="34" t="n">
-        <x:v>46285</x:v>
+        <x:v>46289</x:v>
       </x:c>
       <x:c r="U75" s="13" t="str">
         <x:v>Planned</x:v>
@@ -6587,7 +6606,7 @@
         <x:v>Year-end control check: ✨ NEW — Founder product and lead analytics gives the next operating period cleaner evidence and fewer disconnected handoffs.</x:v>
       </x:c>
       <x:c r="O89" s="13" t="str">
-        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Track first-party signup leads, completed registrations, logins, subscription milestones and throttled module usage in Founder Console without recording passwords, payment secrets or arbitrary clickstreams.</x:v>
+        <x:v>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Track first-party signup leads, completed registrations, logins, subscription milestones and throttled module usage in Founder Console, with retained deleted-state and permanent-removal controls for signup mailing-list entries, without recording passwords, payment secrets or arbitrary clickstreams.</x:v>
       </x:c>
       <x:c r="P89" s="13" t="str">
         <x:v>Prepare your 2027 workflow</x:v>
@@ -6602,7 +6621,7 @@
         <x:v>founder-product-analytics</x:v>
       </x:c>
       <x:c r="T89" s="34" t="n">
-        <x:v>46285</x:v>
+        <x:v>46289</x:v>
       </x:c>
       <x:c r="U89" s="13" t="str">
         <x:v>Planned</x:v>
@@ -6895,7 +6914,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd068d161c98a4a15"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc62767aa109d4140"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7338,10 +7357,14 @@
         <x:v>cashiers, stores, restaurants and walk-in operations</x:v>
       </x:c>
       <x:c r="E22" s="13" t="str">
-        <x:v>Staff can complete counter sales with Cash, direct Transfer or supported terminal payment without opening the wider workspace.</x:v>
-      </x:c>
-      <x:c r="F22" s="13" t="str"/>
-      <x:c r="G22" s="34"/>
+        <x:v>Staff can complete counter sales with Cash, direct Transfer or supported terminal payment only when the tenant plan includes Commerce and Commerce is explicitly enabled; POS still keeps its dedicated user permission.</x:v>
+      </x:c>
+      <x:c r="F22" s="13" t="str">
+        <x:v>NEW</x:v>
+      </x:c>
+      <x:c r="G22" s="34" t="n">
+        <x:v>46289</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="13" t="str">
@@ -7409,7 +7432,7 @@
         <x:v>delivery-notifications</x:v>
       </x:c>
       <x:c r="B26" s="13" t="str">
-        <x:v>Shared realtime Commerce, payment and delivery alert tray</x:v>
+        <x:v>Shared realtime Commerce, Inventory and Finance alert tray</x:v>
       </x:c>
       <x:c r="C26" s="13" t="str">
         <x:v>delivery</x:v>
@@ -7418,13 +7441,13 @@
         <x:v>dispatchers, managers and riders</x:v>
       </x:c>
       <x:c r="E26" s="13" t="str">
-        <x:v>Commerce, payment and Delivery alerts share one movable tray with Inventory without sharing read state; synthesized tones plus eight bundled audio chimes and configurable repeats keep unread work—including direct Transfer verification—hard to miss, while durable Web Push continues due reminders in the background.</x:v>
+        <x:v>Commerce, payment, Delivery, Inventory and Finance attention share one movable access-aware tray without merging their underlying record state; Commerce/Delivery can use durable Web Push in the background, while Finance surfaces unpaid invoices, receivables, payables and balancing anomalies from the same finance records.</x:v>
       </x:c>
       <x:c r="F26" s="13" t="str">
         <x:v>NEW</x:v>
       </x:c>
       <x:c r="G26" s="34" t="n">
-        <x:v>46285</x:v>
+        <x:v>46289</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -7708,13 +7731,13 @@
         <x:v>INPROFIC founders and platform operators</x:v>
       </x:c>
       <x:c r="E40" s="13" t="str">
-        <x:v>Track first-party signup leads, completed registrations, logins, subscription milestones and throttled module usage in Founder Console without recording passwords, payment secrets or arbitrary clickstreams.</x:v>
+        <x:v>Track first-party signup leads, completed registrations, logins, subscription milestones and throttled module usage in Founder Console, with retained deleted-state and permanent-removal controls for signup mailing-list entries, without recording passwords, payment secrets or arbitrary clickstreams.</x:v>
       </x:c>
       <x:c r="F40" s="13" t="str">
         <x:v>NEW</x:v>
       </x:c>
       <x:c r="G40" s="34" t="n">
-        <x:v>46285</x:v>
+        <x:v>46289</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -7794,7 +7817,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c3e60c40e3e4727"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7f0d8b7e4754b9a"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Background Jobs & REDIS Config
</commit_message>
<xml_diff>
--- a/docs/INPROFIC_Q4_2026_Content_Calendar.xlsx
+++ b/docs/INPROFIC_Q4_2026_Content_Calendar.xlsx
@@ -22,8 +22,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -118,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -133,14 +133,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -148,6 +148,11 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -616,7 +621,6 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Campaign phase</t>
@@ -634,9 +638,8 @@
           <t>Scheduled posts</t>
         </is>
       </c>
-      <c r="B4">
-        <f>COUNTA(Calendar!A2:A200)</f>
-        <v/>
+      <c r="B4" t="n">
+        <v>92</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -655,9 +658,8 @@
           <t>Catalogued capabilities</t>
         </is>
       </c>
-      <c r="B5">
-        <f>COUNTA('Feature Catalog'!A2:A200)</f>
-        <v/>
+      <c r="B5" t="n">
+        <v>44</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -676,9 +678,8 @@
           <t>New capabilities highlighted</t>
         </is>
       </c>
-      <c r="B6">
-        <f>COUNTIF('Feature Catalog'!F2:F200,"NEW")</f>
-        <v/>
+      <c r="B6" t="n">
+        <v>17</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -803,7 +804,7 @@
           <t>Raw-material and finished-good warning/low conditions open in separate Inventory tabs inside the movable tray, keep per-user snooze/re-alert timing, can use synthesized alerts or eight bundled audio chimes, and continue due reminders through Web Push when the app is backgrounded or closed.</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="15" t="n">
         <v>46285</v>
       </c>
     </row>
@@ -818,7 +819,7 @@
           <t>Show the business bank account, require customer payment proof externally, and keep payment pending until staff verifies the actual credit.</t>
         </is>
       </c>
-      <c r="C15" s="8" t="n">
+      <c r="C15" s="15" t="n">
         <v>46285</v>
       </c>
     </row>
@@ -833,7 +834,7 @@
           <t>Staff can complete counter sales with Cash, direct Transfer or supported terminal payment only when the tenant plan includes Commerce and Commerce is explicitly enabled; POS still keeps its dedicated user permission.</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
+      <c r="C16" s="15" t="n">
         <v>46289</v>
       </c>
     </row>
@@ -848,7 +849,7 @@
           <t>Keep INPROFIC in control of delivery pricing, routing and tracking while any courier stays manual or connects through a normalized dispatch/status adapter; optional built-in providers remain separately governed.</t>
         </is>
       </c>
-      <c r="C17" s="8" t="n">
+      <c r="C17" s="15" t="n">
         <v>46285</v>
       </c>
     </row>
@@ -863,7 +864,7 @@
           <t>Commerce, payment, Delivery, Inventory and Finance attention share one movable access-aware tray without merging their underlying record state; Commerce/Delivery can use durable Web Push in the background, while Finance surfaces unpaid invoices, receivables, payables and balancing anomalies from the same finance records.</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18" s="15" t="n">
         <v>46289</v>
       </c>
     </row>
@@ -878,7 +879,7 @@
           <t>Control plan pricing, module entitlements, the general free-trial duration and per-business founder trial extensions without deleting tenant history or overlapping active paid/lifetime access.</t>
         </is>
       </c>
-      <c r="C19" s="8" t="n">
+      <c r="C19" s="15" t="n">
         <v>46286</v>
       </c>
     </row>
@@ -893,7 +894,7 @@
           <t>Optional provider connectors can be hidden and execution-blocked platform-wide without deleting tenant credentials or history; businesses still activate their own approved provider accounts only after configuration.</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C20" s="15" t="n">
         <v>46285</v>
       </c>
     </row>
@@ -908,127 +909,142 @@
           <t>Hidden interconnected modules do not stop required back-office synchronization, so upgrades reveal already-complete records.</t>
         </is>
       </c>
-      <c r="C21" s="8" t="n">
+      <c r="C21" s="15" t="n">
         <v>46285</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Surface-safe Online, POS and Distribution pricing</t>
+          <t>Reports, exports and business backup</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Physical Store/direct pricing stays inside the staff POS, while hosted/headless commerce exposes Online plus Distribution/Bulk and INPROFIC enforces the chosen channel and minimum quantity server-side.</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="n">
-        <v>46285</v>
+          <t>Generate a date-range monthly PDF with revenue, sales-origin, procurement, production and inventory charts and tables, alongside exports and a tenant backup.</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="n">
+        <v>46290</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Standard portions, composed products and Bulk Packs</t>
+          <t>Surface-safe Online, POS and Distribution pricing</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Keep production in base units such as scoops/pieces/ml while customers buy plates, servings, bowls, cartons or other packs; show customer-safe package contents and preserve private yield conversions.</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="n">
+          <t>Physical Store/direct pricing stays inside the staff POS, while hosted/headless commerce exposes Online plus Distribution/Bulk and INPROFIC enforces the chosen channel and minimum quantity server-side.</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="n">
         <v>46285</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Founder product and lead analytics</t>
+          <t>Standard portions, composed products and Bulk Packs</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Track first-party signup leads, completed registrations, logins, subscription milestones and throttled module usage in Founder Console, with retained deleted-state and permanent-removal controls for signup mailing-list entries, without recording passwords, payment secrets or arbitrary clickstreams.</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="n">
-        <v>46289</v>
+          <t>Keep production in base units such as scoops/pieces/ml while customers buy plates, servings, bowls, cartons or other packs; show customer-safe package contents and preserve private yield conversions.</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>46285</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Animated, consistent form validation across INPROFIC</t>
+          <t>Founder product and lead analytics</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>HTML5 and Django validation share animated field states, contextual SVG affordances, accessible feedback and consistent toggle switches; dynamic rows inherit the same behavior.</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="n">
-        <v>46285</v>
+          <t>Track first-party signup leads, completed registrations, logins, subscription milestones and throttled module usage in Founder Console, with retained deleted-state and permanent-removal controls for signup mailing-list entries, without recording passwords, payment secrets or arbitrary clickstreams.</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="n">
+        <v>46289</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Channel-aware plain and add-on product options</t>
+          <t>Animated, consistent form validation across INPROFIC</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Offer Extra Jollof, Single Chicken, bottles, pieces or other plain portions from the same Finished Good stock and recipe with independent Physical Store, Online and Bulk/Distribution availability and pricing.</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="n">
+          <t>HTML5 and Django validation share animated field states, contextual SVG affordances, accessible feedback and consistent toggle switches; dynamic rows inherit the same behavior.</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="n">
         <v>46285</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Interactive product demos</t>
+          <t>Channel-aware plain and add-on product options</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>The marketing site provides a vertical-aware workflow, a floating module constellation with flowing brand connectors and viewport-centred previews, plus a detailed storefront-to-fulfilment flow.</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="n">
-        <v>46286</v>
+          <t>Offer Extra Jollof, Single Chicken, bottles, pieces or other plain portions from the same Finished Good stock and recipe with independent Physical Store, Online and Bulk/Distribution availability and pricing.</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="n">
+        <v>46285</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Targeted business mailing workspace</t>
+          <t>Interactive product demos</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Create reusable branded email topics, segment current businesses by service and plan, send immediately, and retry provider failures safely with per-recipient delivery totals.</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="n">
-        <v>46289</v>
+          <t>The marketing site provides a vertical-aware workflow, a floating module constellation with flowing brand connectors and viewport-centred previews, plus a detailed storefront-to-fulfilment flow.</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="n">
+        <v>46286</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
+          <t>Targeted business mailing workspace</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Create reusable branded email topics, segment current businesses by service and plan, send immediately, and retry provider failures safely with per-recipient delivery totals.</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="n">
+        <v>46289</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>Founder-managed trusted-business strip</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>Show a founder-enabled scrolling logo strip above the product demo, automatically limiting tenant logos to paid businesses while the animated platform count includes trials and approved manual logos fill gaps.</t>
         </is>
       </c>
-      <c r="C29" s="8" t="n">
+      <c r="C30" s="16" t="n">
         <v>46290</v>
       </c>
     </row>
@@ -1041,9 +1057,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A9:G9"/>
     <mergeCell ref="A31:H31"/>
     <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A9:G9"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1202,7 +1218,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="n">
+      <c r="A2" s="17" t="n">
         <v>46296</v>
       </c>
       <c r="B2" s="12" t="inlineStr">
@@ -1295,7 +1311,7 @@
           <t>launch</t>
         </is>
       </c>
-      <c r="T2" s="11" t="n">
+      <c r="T2" s="17" t="n">
         <v>46296</v>
       </c>
       <c r="U2" s="12" t="inlineStr">
@@ -1307,7 +1323,7 @@
       <c r="W2" s="12" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="n">
+      <c r="A3" s="17" t="n">
         <v>46297</v>
       </c>
       <c r="B3" s="12" t="inlineStr">
@@ -1400,7 +1416,7 @@
           <t>launch</t>
         </is>
       </c>
-      <c r="T3" s="11" t="n">
+      <c r="T3" s="17" t="n">
         <v>46296</v>
       </c>
       <c r="U3" s="12" t="inlineStr">
@@ -1412,7 +1428,7 @@
       <c r="W3" s="12" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="n">
+      <c r="A4" s="17" t="n">
         <v>46298</v>
       </c>
       <c r="B4" s="12" t="inlineStr">
@@ -1505,7 +1521,7 @@
           <t>launch</t>
         </is>
       </c>
-      <c r="T4" s="11" t="n">
+      <c r="T4" s="17" t="n">
         <v>46296</v>
       </c>
       <c r="U4" s="12" t="inlineStr">
@@ -1517,7 +1533,7 @@
       <c r="W4" s="12" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n">
+      <c r="A5" s="17" t="n">
         <v>46299</v>
       </c>
       <c r="B5" s="12" t="inlineStr">
@@ -1610,7 +1626,7 @@
           <t>launch</t>
         </is>
       </c>
-      <c r="T5" s="11" t="n">
+      <c r="T5" s="17" t="n">
         <v>46296</v>
       </c>
       <c r="U5" s="12" t="inlineStr">
@@ -1622,7 +1638,7 @@
       <c r="W5" s="12" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="n">
+      <c r="A6" s="17" t="n">
         <v>46300</v>
       </c>
       <c r="B6" s="12" t="inlineStr">
@@ -1715,7 +1731,7 @@
           <t>launch</t>
         </is>
       </c>
-      <c r="T6" s="11" t="n">
+      <c r="T6" s="17" t="n">
         <v>46296</v>
       </c>
       <c r="U6" s="12" t="inlineStr">
@@ -1727,7 +1743,7 @@
       <c r="W6" s="12" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n">
+      <c r="A7" s="17" t="n">
         <v>46301</v>
       </c>
       <c r="B7" s="12" t="inlineStr">
@@ -1820,7 +1836,7 @@
           <t>launch</t>
         </is>
       </c>
-      <c r="T7" s="11" t="n">
+      <c r="T7" s="17" t="n">
         <v>46296</v>
       </c>
       <c r="U7" s="12" t="inlineStr">
@@ -1832,7 +1848,7 @@
       <c r="W7" s="12" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="n">
+      <c r="A8" s="17" t="n">
         <v>46302</v>
       </c>
       <c r="B8" s="12" t="inlineStr">
@@ -1925,7 +1941,7 @@
           <t>launch</t>
         </is>
       </c>
-      <c r="T8" s="11" t="n">
+      <c r="T8" s="17" t="n">
         <v>46296</v>
       </c>
       <c r="U8" s="12" t="inlineStr">
@@ -1937,7 +1953,7 @@
       <c r="W8" s="12" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n">
+      <c r="A9" s="17" t="n">
         <v>46303</v>
       </c>
       <c r="B9" s="12" t="inlineStr">
@@ -2026,7 +2042,7 @@
           <t>inventory-units</t>
         </is>
       </c>
-      <c r="T9" s="11" t="inlineStr"/>
+      <c r="T9" s="17" t="inlineStr"/>
       <c r="U9" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -2036,7 +2052,7 @@
       <c r="W9" s="12" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="17" t="n">
         <v>46304</v>
       </c>
       <c r="B10" s="12" t="inlineStr">
@@ -2125,7 +2141,7 @@
           <t>dashboard-insights</t>
         </is>
       </c>
-      <c r="T10" s="11" t="inlineStr"/>
+      <c r="T10" s="17" t="inlineStr"/>
       <c r="U10" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -2135,7 +2151,7 @@
       <c r="W10" s="12" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n">
+      <c r="A11" s="17" t="n">
         <v>46305</v>
       </c>
       <c r="B11" s="12" t="inlineStr">
@@ -2228,7 +2244,7 @@
           <t>stock-alerts</t>
         </is>
       </c>
-      <c r="T11" s="11" t="n">
+      <c r="T11" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U11" s="12" t="inlineStr">
@@ -2240,7 +2256,7 @@
       <c r="W11" s="12" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n">
+      <c r="A12" s="17" t="n">
         <v>46306</v>
       </c>
       <c r="B12" s="12" t="inlineStr">
@@ -2329,7 +2345,7 @@
           <t>product-categories</t>
         </is>
       </c>
-      <c r="T12" s="11" t="inlineStr"/>
+      <c r="T12" s="17" t="inlineStr"/>
       <c r="U12" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -2339,7 +2355,7 @@
       <c r="W12" s="12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n">
+      <c r="A13" s="17" t="n">
         <v>46307</v>
       </c>
       <c r="B13" s="12" t="inlineStr">
@@ -2428,7 +2444,7 @@
           <t>measurement-change</t>
         </is>
       </c>
-      <c r="T13" s="11" t="inlineStr"/>
+      <c r="T13" s="17" t="inlineStr"/>
       <c r="U13" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -2438,7 +2454,7 @@
       <c r="W13" s="12" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n">
+      <c r="A14" s="17" t="n">
         <v>46308</v>
       </c>
       <c r="B14" s="12" t="inlineStr">
@@ -2527,7 +2543,7 @@
           <t>procurement</t>
         </is>
       </c>
-      <c r="T14" s="11" t="inlineStr"/>
+      <c r="T14" s="17" t="inlineStr"/>
       <c r="U14" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -2537,7 +2553,7 @@
       <c r="W14" s="12" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n">
+      <c r="A15" s="17" t="n">
         <v>46309</v>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -2626,7 +2642,7 @@
           <t>wholesale-retail</t>
         </is>
       </c>
-      <c r="T15" s="11" t="inlineStr"/>
+      <c r="T15" s="17" t="inlineStr"/>
       <c r="U15" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -2636,7 +2652,7 @@
       <c r="W15" s="12" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n">
+      <c r="A16" s="17" t="n">
         <v>46310</v>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -2725,7 +2741,7 @@
           <t>production</t>
         </is>
       </c>
-      <c r="T16" s="11" t="inlineStr"/>
+      <c r="T16" s="17" t="inlineStr"/>
       <c r="U16" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -2735,7 +2751,7 @@
       <c r="W16" s="12" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n">
+      <c r="A17" s="17" t="n">
         <v>46311</v>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -2824,7 +2840,7 @@
           <t>shared-runs</t>
         </is>
       </c>
-      <c r="T17" s="11" t="inlineStr"/>
+      <c r="T17" s="17" t="inlineStr"/>
       <c r="U17" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -2834,7 +2850,7 @@
       <c r="W17" s="12" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n">
+      <c r="A18" s="17" t="n">
         <v>46312</v>
       </c>
       <c r="B18" s="12" t="inlineStr">
@@ -2923,7 +2939,7 @@
           <t>batch-yield</t>
         </is>
       </c>
-      <c r="T18" s="11" t="inlineStr"/>
+      <c r="T18" s="17" t="inlineStr"/>
       <c r="U18" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -2933,7 +2949,7 @@
       <c r="W18" s="12" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n">
+      <c r="A19" s="17" t="n">
         <v>46313</v>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -3022,7 +3038,7 @@
           <t>offcuts-shortages</t>
         </is>
       </c>
-      <c r="T19" s="11" t="inlineStr"/>
+      <c r="T19" s="17" t="inlineStr"/>
       <c r="U19" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -3032,7 +3048,7 @@
       <c r="W19" s="12" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n">
+      <c r="A20" s="17" t="n">
         <v>46314</v>
       </c>
       <c r="B20" s="12" t="inlineStr">
@@ -3121,7 +3137,7 @@
           <t>sales</t>
         </is>
       </c>
-      <c r="T20" s="11" t="inlineStr"/>
+      <c r="T20" s="17" t="inlineStr"/>
       <c r="U20" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -3131,7 +3147,7 @@
       <c r="W20" s="12" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="n">
+      <c r="A21" s="17" t="n">
         <v>46315</v>
       </c>
       <c r="B21" s="12" t="inlineStr">
@@ -3220,7 +3236,7 @@
           <t>customer-pricing</t>
         </is>
       </c>
-      <c r="T21" s="11" t="inlineStr"/>
+      <c r="T21" s="17" t="inlineStr"/>
       <c r="U21" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -3230,7 +3246,7 @@
       <c r="W21" s="12" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="n">
+      <c r="A22" s="17" t="n">
         <v>46316</v>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -3319,7 +3335,7 @@
           <t>credit</t>
         </is>
       </c>
-      <c r="T22" s="11" t="inlineStr"/>
+      <c r="T22" s="17" t="inlineStr"/>
       <c r="U22" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -3329,7 +3345,7 @@
       <c r="W22" s="12" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="n">
+      <c r="A23" s="17" t="n">
         <v>46317</v>
       </c>
       <c r="B23" s="12" t="inlineStr">
@@ -3418,7 +3434,7 @@
           <t>finance-ledger</t>
         </is>
       </c>
-      <c r="T23" s="11" t="inlineStr"/>
+      <c r="T23" s="17" t="inlineStr"/>
       <c r="U23" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -3428,7 +3444,7 @@
       <c r="W23" s="12" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="n">
+      <c r="A24" s="17" t="n">
         <v>46318</v>
       </c>
       <c r="B24" s="12" t="inlineStr">
@@ -3517,7 +3533,7 @@
           <t>expenses</t>
         </is>
       </c>
-      <c r="T24" s="11" t="inlineStr"/>
+      <c r="T24" s="17" t="inlineStr"/>
       <c r="U24" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -3527,7 +3543,7 @@
       <c r="W24" s="12" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="n">
+      <c r="A25" s="17" t="n">
         <v>46319</v>
       </c>
       <c r="B25" s="12" t="inlineStr">
@@ -3616,7 +3632,7 @@
           <t>commerce-storefront</t>
         </is>
       </c>
-      <c r="T25" s="11" t="inlineStr"/>
+      <c r="T25" s="17" t="inlineStr"/>
       <c r="U25" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -3626,7 +3642,7 @@
       <c r="W25" s="12" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="n">
+      <c r="A26" s="17" t="n">
         <v>46320</v>
       </c>
       <c r="B26" s="12" t="inlineStr">
@@ -3715,7 +3731,7 @@
           <t>headless-api</t>
         </is>
       </c>
-      <c r="T26" s="11" t="inlineStr"/>
+      <c r="T26" s="17" t="inlineStr"/>
       <c r="U26" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -3725,7 +3741,7 @@
       <c r="W26" s="12" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="n">
+      <c r="A27" s="17" t="n">
         <v>46321</v>
       </c>
       <c r="B27" s="12" t="inlineStr">
@@ -3814,7 +3830,7 @@
           <t>gateway-payments</t>
         </is>
       </c>
-      <c r="T27" s="11" t="inlineStr"/>
+      <c r="T27" s="17" t="inlineStr"/>
       <c r="U27" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -3824,7 +3840,7 @@
       <c r="W27" s="12" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="n">
+      <c r="A28" s="17" t="n">
         <v>46322</v>
       </c>
       <c r="B28" s="12" t="inlineStr">
@@ -3917,7 +3933,7 @@
           <t>direct-transfer</t>
         </is>
       </c>
-      <c r="T28" s="11" t="n">
+      <c r="T28" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U28" s="12" t="inlineStr">
@@ -3929,7 +3945,7 @@
       <c r="W28" s="12" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="n">
+      <c r="A29" s="17" t="n">
         <v>46323</v>
       </c>
       <c r="B29" s="12" t="inlineStr">
@@ -4022,7 +4038,7 @@
           <t>pos</t>
         </is>
       </c>
-      <c r="T29" s="11" t="n">
+      <c r="T29" s="17" t="n">
         <v>46289</v>
       </c>
       <c r="U29" s="12" t="inlineStr">
@@ -4034,7 +4050,7 @@
       <c r="W29" s="12" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="n">
+      <c r="A30" s="17" t="n">
         <v>46324</v>
       </c>
       <c r="B30" s="12" t="inlineStr">
@@ -4123,7 +4139,7 @@
           <t>delivery</t>
         </is>
       </c>
-      <c r="T30" s="11" t="inlineStr"/>
+      <c r="T30" s="17" t="inlineStr"/>
       <c r="U30" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -4133,7 +4149,7 @@
       <c r="W30" s="12" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="n">
+      <c r="A31" s="17" t="n">
         <v>46325</v>
       </c>
       <c r="B31" s="12" t="inlineStr">
@@ -4222,7 +4238,7 @@
           <t>delivery-coverage</t>
         </is>
       </c>
-      <c r="T31" s="11" t="inlineStr"/>
+      <c r="T31" s="17" t="inlineStr"/>
       <c r="U31" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -4232,7 +4248,7 @@
       <c r="W31" s="12" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="n">
+      <c r="A32" s="17" t="n">
         <v>46326</v>
       </c>
       <c r="B32" s="12" t="inlineStr">
@@ -4325,7 +4341,7 @@
           <t>glovo-provider</t>
         </is>
       </c>
-      <c r="T32" s="11" t="n">
+      <c r="T32" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U32" s="12" t="inlineStr">
@@ -4337,7 +4353,7 @@
       <c r="W32" s="12" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="n">
+      <c r="A33" s="17" t="n">
         <v>46327</v>
       </c>
       <c r="B33" s="12" t="inlineStr">
@@ -4430,7 +4446,7 @@
           <t>delivery-notifications</t>
         </is>
       </c>
-      <c r="T33" s="11" t="n">
+      <c r="T33" s="17" t="n">
         <v>46289</v>
       </c>
       <c r="U33" s="12" t="inlineStr">
@@ -4442,7 +4458,7 @@
       <c r="W33" s="12" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="n">
+      <c r="A34" s="17" t="n">
         <v>46328</v>
       </c>
       <c r="B34" s="12" t="inlineStr">
@@ -4531,7 +4547,7 @@
           <t>rider</t>
         </is>
       </c>
-      <c r="T34" s="11" t="inlineStr"/>
+      <c r="T34" s="17" t="inlineStr"/>
       <c r="U34" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -4541,7 +4557,7 @@
       <c r="W34" s="12" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="n">
+      <c r="A35" s="17" t="n">
         <v>46329</v>
       </c>
       <c r="B35" s="12" t="inlineStr">
@@ -4630,7 +4646,7 @@
           <t>customer-profiles</t>
         </is>
       </c>
-      <c r="T35" s="11" t="inlineStr"/>
+      <c r="T35" s="17" t="inlineStr"/>
       <c r="U35" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -4640,7 +4656,7 @@
       <c r="W35" s="12" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="n">
+      <c r="A36" s="17" t="n">
         <v>46330</v>
       </c>
       <c r="B36" s="12" t="inlineStr">
@@ -4729,7 +4745,7 @@
           <t>audit</t>
         </is>
       </c>
-      <c r="T36" s="11" t="inlineStr"/>
+      <c r="T36" s="17" t="inlineStr"/>
       <c r="U36" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -4739,7 +4755,7 @@
       <c r="W36" s="12" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="n">
+      <c r="A37" s="17" t="n">
         <v>46331</v>
       </c>
       <c r="B37" s="12" t="inlineStr">
@@ -4828,7 +4844,7 @@
           <t>roles</t>
         </is>
       </c>
-      <c r="T37" s="11" t="inlineStr"/>
+      <c r="T37" s="17" t="inlineStr"/>
       <c r="U37" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -4838,7 +4854,7 @@
       <c r="W37" s="12" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="n">
+      <c r="A38" s="17" t="n">
         <v>46332</v>
       </c>
       <c r="B38" s="12" t="inlineStr">
@@ -4927,7 +4943,7 @@
           <t>workspace-theming</t>
         </is>
       </c>
-      <c r="T38" s="11" t="inlineStr"/>
+      <c r="T38" s="17" t="inlineStr"/>
       <c r="U38" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -4937,7 +4953,7 @@
       <c r="W38" s="12" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="n">
+      <c r="A39" s="17" t="n">
         <v>46333</v>
       </c>
       <c r="B39" s="12" t="inlineStr">
@@ -5030,7 +5046,7 @@
           <t>subscriptions</t>
         </is>
       </c>
-      <c r="T39" s="11" t="n">
+      <c r="T39" s="17" t="n">
         <v>46286</v>
       </c>
       <c r="U39" s="12" t="inlineStr">
@@ -5042,7 +5058,7 @@
       <c r="W39" s="12" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="n">
+      <c r="A40" s="17" t="n">
         <v>46334</v>
       </c>
       <c r="B40" s="12" t="inlineStr">
@@ -5135,7 +5151,7 @@
           <t>founder-integration-gates</t>
         </is>
       </c>
-      <c r="T40" s="11" t="n">
+      <c r="T40" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U40" s="12" t="inlineStr">
@@ -5147,7 +5163,7 @@
       <c r="W40" s="12" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="n">
+      <c r="A41" s="17" t="n">
         <v>46335</v>
       </c>
       <c r="B41" s="12" t="inlineStr">
@@ -5236,7 +5252,7 @@
           <t>multi-service-profiles</t>
         </is>
       </c>
-      <c r="T41" s="11" t="inlineStr"/>
+      <c r="T41" s="17" t="inlineStr"/>
       <c r="U41" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -5246,7 +5262,7 @@
       <c r="W41" s="12" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="11" t="n">
+      <c r="A42" s="17" t="n">
         <v>46336</v>
       </c>
       <c r="B42" s="12" t="inlineStr">
@@ -5339,7 +5355,7 @@
           <t>entitlement-continuity</t>
         </is>
       </c>
-      <c r="T42" s="11" t="n">
+      <c r="T42" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U42" s="12" t="inlineStr">
@@ -5351,7 +5367,7 @@
       <c r="W42" s="12" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="n">
+      <c r="A43" s="17" t="n">
         <v>46337</v>
       </c>
       <c r="B43" s="12" t="inlineStr">
@@ -5386,7 +5402,7 @@
       </c>
       <c r="H43" s="12" t="inlineStr">
         <is>
-          <t>Reports, exports and business backup</t>
+          <t>✨ NEW — Reports, exports and business backup</t>
         </is>
       </c>
       <c r="I43" s="12" t="inlineStr">
@@ -5416,12 +5432,12 @@
       </c>
       <c r="N43" s="12" t="inlineStr">
         <is>
-          <t>Still solving this manually? Reports, exports and business backup keeps the workflow connected instead of handing it off to another spreadsheet.</t>
+          <t>Still solving this manually? ✨ NEW — Reports, exports and business backup keeps the workflow connected instead of handing it off to another spreadsheet.</t>
         </is>
       </c>
       <c r="O43" s="12" t="inlineStr">
         <is>
-          <t>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Export operational reports and maintain a tenant backup path without flattening audit history.</t>
+          <t>Start from a familiar operational problem, then show the INPROFIC workflow that resolves it. Proof point: Generate a date-range monthly PDF with revenue, sales-origin, procurement, production and inventory charts and tables, alongside exports and a tenant backup.</t>
         </is>
       </c>
       <c r="P43" s="12" t="inlineStr">
@@ -5434,13 +5450,19 @@
           <t>Use a real INPROFIC screen/demo for Reports, exports and business backup. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</t>
         </is>
       </c>
-      <c r="R43" s="12" t="inlineStr"/>
+      <c r="R43" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="S43" s="12" t="inlineStr">
         <is>
           <t>reports-backup</t>
         </is>
       </c>
-      <c r="T43" s="11" t="inlineStr"/>
+      <c r="T43" s="17" t="n">
+        <v>46290</v>
+      </c>
       <c r="U43" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -5450,7 +5472,7 @@
       <c r="W43" s="12" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="11" t="n">
+      <c r="A44" s="17" t="n">
         <v>46338</v>
       </c>
       <c r="B44" s="12" t="inlineStr">
@@ -5539,7 +5561,7 @@
           <t>onboarding</t>
         </is>
       </c>
-      <c r="T44" s="11" t="inlineStr"/>
+      <c r="T44" s="17" t="inlineStr"/>
       <c r="U44" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -5549,7 +5571,7 @@
       <c r="W44" s="12" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="11" t="n">
+      <c r="A45" s="17" t="n">
         <v>46339</v>
       </c>
       <c r="B45" s="12" t="inlineStr">
@@ -5642,7 +5664,7 @@
           <t>commerce-channel-boundary</t>
         </is>
       </c>
-      <c r="T45" s="11" t="n">
+      <c r="T45" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U45" s="12" t="inlineStr">
@@ -5654,7 +5676,7 @@
       <c r="W45" s="12" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="11" t="n">
+      <c r="A46" s="17" t="n">
         <v>46340</v>
       </c>
       <c r="B46" s="12" t="inlineStr">
@@ -5747,7 +5769,7 @@
           <t>portion-bulk-pack-composition</t>
         </is>
       </c>
-      <c r="T46" s="11" t="n">
+      <c r="T46" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U46" s="12" t="inlineStr">
@@ -5759,7 +5781,7 @@
       <c r="W46" s="12" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="11" t="n">
+      <c r="A47" s="17" t="n">
         <v>46341</v>
       </c>
       <c r="B47" s="12" t="inlineStr">
@@ -5852,7 +5874,7 @@
           <t>founder-product-analytics</t>
         </is>
       </c>
-      <c r="T47" s="11" t="n">
+      <c r="T47" s="17" t="n">
         <v>46289</v>
       </c>
       <c r="U47" s="12" t="inlineStr">
@@ -5864,7 +5886,7 @@
       <c r="W47" s="12" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="11" t="n">
+      <c r="A48" s="17" t="n">
         <v>46342</v>
       </c>
       <c r="B48" s="12" t="inlineStr">
@@ -5957,7 +5979,7 @@
           <t>form-experience-v2</t>
         </is>
       </c>
-      <c r="T48" s="11" t="n">
+      <c r="T48" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U48" s="12" t="inlineStr">
@@ -5969,7 +5991,7 @@
       <c r="W48" s="12" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="11" t="n">
+      <c r="A49" s="17" t="n">
         <v>46343</v>
       </c>
       <c r="B49" s="12" t="inlineStr">
@@ -6062,7 +6084,7 @@
           <t>individual-sale-options</t>
         </is>
       </c>
-      <c r="T49" s="11" t="n">
+      <c r="T49" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U49" s="12" t="inlineStr">
@@ -6074,7 +6096,7 @@
       <c r="W49" s="12" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="11" t="n">
+      <c r="A50" s="17" t="n">
         <v>46344</v>
       </c>
       <c r="B50" s="12" t="inlineStr">
@@ -6167,7 +6189,7 @@
           <t>interactive-product-demos</t>
         </is>
       </c>
-      <c r="T50" s="11" t="n">
+      <c r="T50" s="17" t="n">
         <v>46286</v>
       </c>
       <c r="U50" s="12" t="inlineStr">
@@ -6179,7 +6201,7 @@
       <c r="W50" s="12" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="11" t="n">
+      <c r="A51" s="17" t="n">
         <v>46345</v>
       </c>
       <c r="B51" s="12" t="inlineStr">
@@ -6272,7 +6294,7 @@
           <t>platform-mailing-workspace</t>
         </is>
       </c>
-      <c r="T51" s="11" t="n">
+      <c r="T51" s="17" t="n">
         <v>46289</v>
       </c>
       <c r="U51" s="12" t="inlineStr">
@@ -6284,7 +6306,7 @@
       <c r="W51" s="12" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="11" t="n">
+      <c r="A52" s="17" t="n">
         <v>46346</v>
       </c>
       <c r="B52" s="12" t="inlineStr">
@@ -6377,7 +6399,7 @@
           <t>trusted-business-strip</t>
         </is>
       </c>
-      <c r="T52" s="11" t="n">
+      <c r="T52" s="17" t="n">
         <v>46290</v>
       </c>
       <c r="U52" s="12" t="inlineStr">
@@ -6389,7 +6411,7 @@
       <c r="W52" s="12" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="11" t="n">
+      <c r="A53" s="17" t="n">
         <v>46347</v>
       </c>
       <c r="B53" s="12" t="inlineStr">
@@ -6478,7 +6500,7 @@
           <t>inventory-units</t>
         </is>
       </c>
-      <c r="T53" s="11" t="inlineStr"/>
+      <c r="T53" s="17" t="inlineStr"/>
       <c r="U53" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -6488,7 +6510,7 @@
       <c r="W53" s="12" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="11" t="n">
+      <c r="A54" s="17" t="n">
         <v>46348</v>
       </c>
       <c r="B54" s="12" t="inlineStr">
@@ -6577,7 +6599,7 @@
           <t>dashboard-insights</t>
         </is>
       </c>
-      <c r="T54" s="11" t="inlineStr"/>
+      <c r="T54" s="17" t="inlineStr"/>
       <c r="U54" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -6587,7 +6609,7 @@
       <c r="W54" s="12" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="11" t="n">
+      <c r="A55" s="17" t="n">
         <v>46349</v>
       </c>
       <c r="B55" s="12" t="inlineStr">
@@ -6680,7 +6702,7 @@
           <t>stock-alerts</t>
         </is>
       </c>
-      <c r="T55" s="11" t="n">
+      <c r="T55" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U55" s="12" t="inlineStr">
@@ -6692,7 +6714,7 @@
       <c r="W55" s="12" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="11" t="n">
+      <c r="A56" s="17" t="n">
         <v>46350</v>
       </c>
       <c r="B56" s="12" t="inlineStr">
@@ -6781,7 +6803,7 @@
           <t>product-categories</t>
         </is>
       </c>
-      <c r="T56" s="11" t="inlineStr"/>
+      <c r="T56" s="17" t="inlineStr"/>
       <c r="U56" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -6791,7 +6813,7 @@
       <c r="W56" s="12" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="11" t="n">
+      <c r="A57" s="17" t="n">
         <v>46351</v>
       </c>
       <c r="B57" s="12" t="inlineStr">
@@ -6880,7 +6902,7 @@
           <t>measurement-change</t>
         </is>
       </c>
-      <c r="T57" s="11" t="inlineStr"/>
+      <c r="T57" s="17" t="inlineStr"/>
       <c r="U57" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -6890,7 +6912,7 @@
       <c r="W57" s="12" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="11" t="n">
+      <c r="A58" s="17" t="n">
         <v>46352</v>
       </c>
       <c r="B58" s="12" t="inlineStr">
@@ -6979,7 +7001,7 @@
           <t>procurement</t>
         </is>
       </c>
-      <c r="T58" s="11" t="inlineStr"/>
+      <c r="T58" s="17" t="inlineStr"/>
       <c r="U58" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -6989,7 +7011,7 @@
       <c r="W58" s="12" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="n">
+      <c r="A59" s="17" t="n">
         <v>46353</v>
       </c>
       <c r="B59" s="12" t="inlineStr">
@@ -7078,7 +7100,7 @@
           <t>wholesale-retail</t>
         </is>
       </c>
-      <c r="T59" s="11" t="inlineStr"/>
+      <c r="T59" s="17" t="inlineStr"/>
       <c r="U59" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -7088,7 +7110,7 @@
       <c r="W59" s="12" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="11" t="n">
+      <c r="A60" s="17" t="n">
         <v>46354</v>
       </c>
       <c r="B60" s="12" t="inlineStr">
@@ -7177,7 +7199,7 @@
           <t>production</t>
         </is>
       </c>
-      <c r="T60" s="11" t="inlineStr"/>
+      <c r="T60" s="17" t="inlineStr"/>
       <c r="U60" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -7187,7 +7209,7 @@
       <c r="W60" s="12" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="11" t="n">
+      <c r="A61" s="17" t="n">
         <v>46355</v>
       </c>
       <c r="B61" s="12" t="inlineStr">
@@ -7276,7 +7298,7 @@
           <t>shared-runs</t>
         </is>
       </c>
-      <c r="T61" s="11" t="inlineStr"/>
+      <c r="T61" s="17" t="inlineStr"/>
       <c r="U61" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -7286,7 +7308,7 @@
       <c r="W61" s="12" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="11" t="n">
+      <c r="A62" s="17" t="n">
         <v>46356</v>
       </c>
       <c r="B62" s="12" t="inlineStr">
@@ -7375,7 +7397,7 @@
           <t>batch-yield</t>
         </is>
       </c>
-      <c r="T62" s="11" t="inlineStr"/>
+      <c r="T62" s="17" t="inlineStr"/>
       <c r="U62" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -7385,7 +7407,7 @@
       <c r="W62" s="12" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="11" t="n">
+      <c r="A63" s="17" t="n">
         <v>46357</v>
       </c>
       <c r="B63" s="12" t="inlineStr">
@@ -7474,7 +7496,7 @@
           <t>offcuts-shortages</t>
         </is>
       </c>
-      <c r="T63" s="11" t="inlineStr"/>
+      <c r="T63" s="17" t="inlineStr"/>
       <c r="U63" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -7484,7 +7506,7 @@
       <c r="W63" s="12" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="11" t="n">
+      <c r="A64" s="17" t="n">
         <v>46358</v>
       </c>
       <c r="B64" s="12" t="inlineStr">
@@ -7573,7 +7595,7 @@
           <t>sales</t>
         </is>
       </c>
-      <c r="T64" s="11" t="inlineStr"/>
+      <c r="T64" s="17" t="inlineStr"/>
       <c r="U64" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -7583,7 +7605,7 @@
       <c r="W64" s="12" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="11" t="n">
+      <c r="A65" s="17" t="n">
         <v>46359</v>
       </c>
       <c r="B65" s="12" t="inlineStr">
@@ -7672,7 +7694,7 @@
           <t>customer-pricing</t>
         </is>
       </c>
-      <c r="T65" s="11" t="inlineStr"/>
+      <c r="T65" s="17" t="inlineStr"/>
       <c r="U65" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -7682,7 +7704,7 @@
       <c r="W65" s="12" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="11" t="n">
+      <c r="A66" s="17" t="n">
         <v>46360</v>
       </c>
       <c r="B66" s="12" t="inlineStr">
@@ -7771,7 +7793,7 @@
           <t>credit</t>
         </is>
       </c>
-      <c r="T66" s="11" t="inlineStr"/>
+      <c r="T66" s="17" t="inlineStr"/>
       <c r="U66" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -7781,7 +7803,7 @@
       <c r="W66" s="12" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="11" t="n">
+      <c r="A67" s="17" t="n">
         <v>46361</v>
       </c>
       <c r="B67" s="12" t="inlineStr">
@@ -7870,7 +7892,7 @@
           <t>finance-ledger</t>
         </is>
       </c>
-      <c r="T67" s="11" t="inlineStr"/>
+      <c r="T67" s="17" t="inlineStr"/>
       <c r="U67" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -7880,7 +7902,7 @@
       <c r="W67" s="12" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="11" t="n">
+      <c r="A68" s="17" t="n">
         <v>46362</v>
       </c>
       <c r="B68" s="12" t="inlineStr">
@@ -7969,7 +7991,7 @@
           <t>expenses</t>
         </is>
       </c>
-      <c r="T68" s="11" t="inlineStr"/>
+      <c r="T68" s="17" t="inlineStr"/>
       <c r="U68" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -7979,7 +8001,7 @@
       <c r="W68" s="12" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="11" t="n">
+      <c r="A69" s="17" t="n">
         <v>46363</v>
       </c>
       <c r="B69" s="12" t="inlineStr">
@@ -8068,7 +8090,7 @@
           <t>commerce-storefront</t>
         </is>
       </c>
-      <c r="T69" s="11" t="inlineStr"/>
+      <c r="T69" s="17" t="inlineStr"/>
       <c r="U69" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -8078,7 +8100,7 @@
       <c r="W69" s="12" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="11" t="n">
+      <c r="A70" s="17" t="n">
         <v>46364</v>
       </c>
       <c r="B70" s="12" t="inlineStr">
@@ -8167,7 +8189,7 @@
           <t>headless-api</t>
         </is>
       </c>
-      <c r="T70" s="11" t="inlineStr"/>
+      <c r="T70" s="17" t="inlineStr"/>
       <c r="U70" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -8177,7 +8199,7 @@
       <c r="W70" s="12" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="11" t="n">
+      <c r="A71" s="17" t="n">
         <v>46365</v>
       </c>
       <c r="B71" s="12" t="inlineStr">
@@ -8266,7 +8288,7 @@
           <t>gateway-payments</t>
         </is>
       </c>
-      <c r="T71" s="11" t="inlineStr"/>
+      <c r="T71" s="17" t="inlineStr"/>
       <c r="U71" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -8276,7 +8298,7 @@
       <c r="W71" s="12" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="11" t="n">
+      <c r="A72" s="17" t="n">
         <v>46366</v>
       </c>
       <c r="B72" s="12" t="inlineStr">
@@ -8369,7 +8391,7 @@
           <t>direct-transfer</t>
         </is>
       </c>
-      <c r="T72" s="11" t="n">
+      <c r="T72" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U72" s="12" t="inlineStr">
@@ -8381,7 +8403,7 @@
       <c r="W72" s="12" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="11" t="n">
+      <c r="A73" s="17" t="n">
         <v>46367</v>
       </c>
       <c r="B73" s="12" t="inlineStr">
@@ -8474,7 +8496,7 @@
           <t>pos</t>
         </is>
       </c>
-      <c r="T73" s="11" t="n">
+      <c r="T73" s="17" t="n">
         <v>46289</v>
       </c>
       <c r="U73" s="12" t="inlineStr">
@@ -8486,7 +8508,7 @@
       <c r="W73" s="12" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="11" t="n">
+      <c r="A74" s="17" t="n">
         <v>46368</v>
       </c>
       <c r="B74" s="12" t="inlineStr">
@@ -8575,7 +8597,7 @@
           <t>delivery</t>
         </is>
       </c>
-      <c r="T74" s="11" t="inlineStr"/>
+      <c r="T74" s="17" t="inlineStr"/>
       <c r="U74" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -8585,7 +8607,7 @@
       <c r="W74" s="12" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="11" t="n">
+      <c r="A75" s="17" t="n">
         <v>46369</v>
       </c>
       <c r="B75" s="12" t="inlineStr">
@@ -8674,7 +8696,7 @@
           <t>delivery-coverage</t>
         </is>
       </c>
-      <c r="T75" s="11" t="inlineStr"/>
+      <c r="T75" s="17" t="inlineStr"/>
       <c r="U75" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -8684,7 +8706,7 @@
       <c r="W75" s="12" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="11" t="n">
+      <c r="A76" s="17" t="n">
         <v>46370</v>
       </c>
       <c r="B76" s="12" t="inlineStr">
@@ -8777,7 +8799,7 @@
           <t>glovo-provider</t>
         </is>
       </c>
-      <c r="T76" s="11" t="n">
+      <c r="T76" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U76" s="12" t="inlineStr">
@@ -8789,7 +8811,7 @@
       <c r="W76" s="12" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="11" t="n">
+      <c r="A77" s="17" t="n">
         <v>46371</v>
       </c>
       <c r="B77" s="12" t="inlineStr">
@@ -8882,7 +8904,7 @@
           <t>delivery-notifications</t>
         </is>
       </c>
-      <c r="T77" s="11" t="n">
+      <c r="T77" s="17" t="n">
         <v>46289</v>
       </c>
       <c r="U77" s="12" t="inlineStr">
@@ -8894,7 +8916,7 @@
       <c r="W77" s="12" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="11" t="n">
+      <c r="A78" s="17" t="n">
         <v>46372</v>
       </c>
       <c r="B78" s="12" t="inlineStr">
@@ -8983,7 +9005,7 @@
           <t>rider</t>
         </is>
       </c>
-      <c r="T78" s="11" t="inlineStr"/>
+      <c r="T78" s="17" t="inlineStr"/>
       <c r="U78" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -8993,7 +9015,7 @@
       <c r="W78" s="12" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="11" t="n">
+      <c r="A79" s="17" t="n">
         <v>46373</v>
       </c>
       <c r="B79" s="12" t="inlineStr">
@@ -9082,7 +9104,7 @@
           <t>customer-profiles</t>
         </is>
       </c>
-      <c r="T79" s="11" t="inlineStr"/>
+      <c r="T79" s="17" t="inlineStr"/>
       <c r="U79" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -9092,7 +9114,7 @@
       <c r="W79" s="12" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="11" t="n">
+      <c r="A80" s="17" t="n">
         <v>46374</v>
       </c>
       <c r="B80" s="12" t="inlineStr">
@@ -9181,7 +9203,7 @@
           <t>audit</t>
         </is>
       </c>
-      <c r="T80" s="11" t="inlineStr"/>
+      <c r="T80" s="17" t="inlineStr"/>
       <c r="U80" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -9191,7 +9213,7 @@
       <c r="W80" s="12" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="11" t="n">
+      <c r="A81" s="17" t="n">
         <v>46375</v>
       </c>
       <c r="B81" s="12" t="inlineStr">
@@ -9280,7 +9302,7 @@
           <t>roles</t>
         </is>
       </c>
-      <c r="T81" s="11" t="inlineStr"/>
+      <c r="T81" s="17" t="inlineStr"/>
       <c r="U81" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -9290,7 +9312,7 @@
       <c r="W81" s="12" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="11" t="n">
+      <c r="A82" s="17" t="n">
         <v>46376</v>
       </c>
       <c r="B82" s="12" t="inlineStr">
@@ -9379,7 +9401,7 @@
           <t>workspace-theming</t>
         </is>
       </c>
-      <c r="T82" s="11" t="inlineStr"/>
+      <c r="T82" s="17" t="inlineStr"/>
       <c r="U82" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -9389,7 +9411,7 @@
       <c r="W82" s="12" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="11" t="n">
+      <c r="A83" s="17" t="n">
         <v>46377</v>
       </c>
       <c r="B83" s="12" t="inlineStr">
@@ -9482,7 +9504,7 @@
           <t>subscriptions</t>
         </is>
       </c>
-      <c r="T83" s="11" t="n">
+      <c r="T83" s="17" t="n">
         <v>46286</v>
       </c>
       <c r="U83" s="12" t="inlineStr">
@@ -9494,7 +9516,7 @@
       <c r="W83" s="12" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="11" t="n">
+      <c r="A84" s="17" t="n">
         <v>46378</v>
       </c>
       <c r="B84" s="12" t="inlineStr">
@@ -9587,7 +9609,7 @@
           <t>founder-integration-gates</t>
         </is>
       </c>
-      <c r="T84" s="11" t="n">
+      <c r="T84" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U84" s="12" t="inlineStr">
@@ -9599,7 +9621,7 @@
       <c r="W84" s="12" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="11" t="n">
+      <c r="A85" s="17" t="n">
         <v>46379</v>
       </c>
       <c r="B85" s="12" t="inlineStr">
@@ -9688,7 +9710,7 @@
           <t>multi-service-profiles</t>
         </is>
       </c>
-      <c r="T85" s="11" t="inlineStr"/>
+      <c r="T85" s="17" t="inlineStr"/>
       <c r="U85" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -9698,7 +9720,7 @@
       <c r="W85" s="12" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="11" t="n">
+      <c r="A86" s="17" t="n">
         <v>46380</v>
       </c>
       <c r="B86" s="12" t="inlineStr">
@@ -9791,7 +9813,7 @@
           <t>entitlement-continuity</t>
         </is>
       </c>
-      <c r="T86" s="11" t="n">
+      <c r="T86" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U86" s="12" t="inlineStr">
@@ -9803,7 +9825,7 @@
       <c r="W86" s="12" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="11" t="n">
+      <c r="A87" s="17" t="n">
         <v>46381</v>
       </c>
       <c r="B87" s="12" t="inlineStr">
@@ -9838,7 +9860,7 @@
       </c>
       <c r="H87" s="12" t="inlineStr">
         <is>
-          <t>Reports, exports and business backup</t>
+          <t>✨ NEW — Reports, exports and business backup</t>
         </is>
       </c>
       <c r="I87" s="12" t="inlineStr">
@@ -9868,12 +9890,12 @@
       </c>
       <c r="N87" s="12" t="inlineStr">
         <is>
-          <t>Year-end control check: Reports, exports and business backup gives the next operating period cleaner evidence and fewer disconnected handoffs.</t>
+          <t>Year-end control check: ✨ NEW — Reports, exports and business backup gives the next operating period cleaner evidence and fewer disconnected handoffs.</t>
         </is>
       </c>
       <c r="O87" s="12" t="inlineStr">
         <is>
-          <t>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Export operational reports and maintain a tenant backup path without flattening audit history.</t>
+          <t>Frame the feature around cleaner controls, fewer manual gaps and readiness for the next operating period without inventing savings claims. Proof point: Generate a date-range monthly PDF with revenue, sales-origin, procurement, production and inventory charts and tables, alongside exports and a tenant backup.</t>
         </is>
       </c>
       <c r="P87" s="12" t="inlineStr">
@@ -9886,13 +9908,19 @@
           <t>Use a real INPROFIC screen/demo for Reports, exports and business backup. Show one before/after workflow, then one concrete proof point; avoid fabricated metrics.</t>
         </is>
       </c>
-      <c r="R87" s="12" t="inlineStr"/>
+      <c r="R87" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="S87" s="12" t="inlineStr">
         <is>
           <t>reports-backup</t>
         </is>
       </c>
-      <c r="T87" s="11" t="inlineStr"/>
+      <c r="T87" s="17" t="n">
+        <v>46290</v>
+      </c>
       <c r="U87" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -9902,7 +9930,7 @@
       <c r="W87" s="12" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="11" t="n">
+      <c r="A88" s="17" t="n">
         <v>46382</v>
       </c>
       <c r="B88" s="12" t="inlineStr">
@@ -9991,7 +10019,7 @@
           <t>onboarding</t>
         </is>
       </c>
-      <c r="T88" s="11" t="inlineStr"/>
+      <c r="T88" s="17" t="inlineStr"/>
       <c r="U88" s="12" t="inlineStr">
         <is>
           <t>Planned</t>
@@ -10001,7 +10029,7 @@
       <c r="W88" s="12" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="11" t="n">
+      <c r="A89" s="17" t="n">
         <v>46383</v>
       </c>
       <c r="B89" s="12" t="inlineStr">
@@ -10094,7 +10122,7 @@
           <t>commerce-channel-boundary</t>
         </is>
       </c>
-      <c r="T89" s="11" t="n">
+      <c r="T89" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U89" s="12" t="inlineStr">
@@ -10106,7 +10134,7 @@
       <c r="W89" s="12" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="11" t="n">
+      <c r="A90" s="17" t="n">
         <v>46384</v>
       </c>
       <c r="B90" s="12" t="inlineStr">
@@ -10199,7 +10227,7 @@
           <t>portion-bulk-pack-composition</t>
         </is>
       </c>
-      <c r="T90" s="11" t="n">
+      <c r="T90" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U90" s="12" t="inlineStr">
@@ -10211,7 +10239,7 @@
       <c r="W90" s="12" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="11" t="n">
+      <c r="A91" s="17" t="n">
         <v>46385</v>
       </c>
       <c r="B91" s="12" t="inlineStr">
@@ -10304,7 +10332,7 @@
           <t>founder-product-analytics</t>
         </is>
       </c>
-      <c r="T91" s="11" t="n">
+      <c r="T91" s="17" t="n">
         <v>46289</v>
       </c>
       <c r="U91" s="12" t="inlineStr">
@@ -10316,7 +10344,7 @@
       <c r="W91" s="12" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="11" t="n">
+      <c r="A92" s="17" t="n">
         <v>46386</v>
       </c>
       <c r="B92" s="12" t="inlineStr">
@@ -10409,7 +10437,7 @@
           <t>form-experience-v2</t>
         </is>
       </c>
-      <c r="T92" s="11" t="n">
+      <c r="T92" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U92" s="12" t="inlineStr">
@@ -10421,7 +10449,7 @@
       <c r="W92" s="12" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" s="11" t="n">
+      <c r="A93" s="17" t="n">
         <v>46387</v>
       </c>
       <c r="B93" s="12" t="inlineStr">
@@ -10514,7 +10542,7 @@
           <t>individual-sale-options</t>
         </is>
       </c>
-      <c r="T93" s="11" t="n">
+      <c r="T93" s="17" t="n">
         <v>46285</v>
       </c>
       <c r="U93" s="12" t="inlineStr">
@@ -10626,7 +10654,7 @@
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr"/>
-      <c r="G2" s="11" t="n"/>
+      <c r="G2" s="17" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -10655,7 +10683,7 @@
         </is>
       </c>
       <c r="F3" s="12" t="inlineStr"/>
-      <c r="G3" s="11" t="n"/>
+      <c r="G3" s="17" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -10688,7 +10716,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
+      <c r="G4" s="17" t="n">
         <v>46285</v>
       </c>
     </row>
@@ -10719,7 +10747,7 @@
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr"/>
-      <c r="G5" s="11" t="n"/>
+      <c r="G5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -10748,7 +10776,7 @@
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr"/>
-      <c r="G6" s="11" t="n"/>
+      <c r="G6" s="17" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -10777,7 +10805,7 @@
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr"/>
-      <c r="G7" s="11" t="n"/>
+      <c r="G7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -10806,7 +10834,7 @@
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr"/>
-      <c r="G8" s="11" t="n"/>
+      <c r="G8" s="17" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -10835,7 +10863,7 @@
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr"/>
-      <c r="G9" s="11" t="n"/>
+      <c r="G9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -10864,7 +10892,7 @@
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr"/>
-      <c r="G10" s="11" t="n"/>
+      <c r="G10" s="17" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -10893,7 +10921,7 @@
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr"/>
-      <c r="G11" s="11" t="n"/>
+      <c r="G11" s="17" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -10922,7 +10950,7 @@
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr"/>
-      <c r="G12" s="11" t="n"/>
+      <c r="G12" s="17" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
@@ -10951,7 +10979,7 @@
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr"/>
-      <c r="G13" s="11" t="n"/>
+      <c r="G13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -10980,7 +11008,7 @@
         </is>
       </c>
       <c r="F14" s="12" t="inlineStr"/>
-      <c r="G14" s="11" t="n"/>
+      <c r="G14" s="17" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -11009,7 +11037,7 @@
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="G15" s="17" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -11038,7 +11066,7 @@
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr"/>
-      <c r="G16" s="11" t="n"/>
+      <c r="G16" s="17" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
@@ -11067,7 +11095,7 @@
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr"/>
-      <c r="G17" s="11" t="n"/>
+      <c r="G17" s="17" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
@@ -11096,7 +11124,7 @@
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr"/>
-      <c r="G18" s="11" t="n"/>
+      <c r="G18" s="17" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
@@ -11125,7 +11153,7 @@
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="G19" s="17" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -11154,7 +11182,7 @@
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr"/>
-      <c r="G20" s="11" t="n"/>
+      <c r="G20" s="17" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
@@ -11187,7 +11215,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
+      <c r="G21" s="17" t="n">
         <v>46285</v>
       </c>
     </row>
@@ -11222,7 +11250,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
+      <c r="G22" s="17" t="n">
         <v>46289</v>
       </c>
     </row>
@@ -11253,7 +11281,7 @@
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr"/>
-      <c r="G23" s="11" t="n"/>
+      <c r="G23" s="17" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
@@ -11282,7 +11310,7 @@
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr"/>
-      <c r="G24" s="11" t="n"/>
+      <c r="G24" s="17" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
@@ -11315,7 +11343,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G25" s="11" t="n">
+      <c r="G25" s="17" t="n">
         <v>46285</v>
       </c>
     </row>
@@ -11350,7 +11378,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G26" s="11" t="n">
+      <c r="G26" s="17" t="n">
         <v>46289</v>
       </c>
     </row>
@@ -11381,7 +11409,7 @@
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr"/>
-      <c r="G27" s="11" t="n"/>
+      <c r="G27" s="17" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
@@ -11410,7 +11438,7 @@
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr"/>
-      <c r="G28" s="11" t="n"/>
+      <c r="G28" s="17" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
@@ -11439,7 +11467,7 @@
         </is>
       </c>
       <c r="F29" s="12" t="inlineStr"/>
-      <c r="G29" s="11" t="n"/>
+      <c r="G29" s="17" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
@@ -11468,7 +11496,7 @@
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr"/>
-      <c r="G30" s="11" t="n"/>
+      <c r="G30" s="17" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
@@ -11497,7 +11525,7 @@
         </is>
       </c>
       <c r="F31" s="12" t="inlineStr"/>
-      <c r="G31" s="11" t="n"/>
+      <c r="G31" s="17" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
@@ -11530,7 +11558,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G32" s="11" t="n">
+      <c r="G32" s="17" t="n">
         <v>46286</v>
       </c>
     </row>
@@ -11565,7 +11593,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G33" s="11" t="n">
+      <c r="G33" s="17" t="n">
         <v>46285</v>
       </c>
     </row>
@@ -11596,7 +11624,7 @@
         </is>
       </c>
       <c r="F34" s="12" t="inlineStr"/>
-      <c r="G34" s="11" t="n"/>
+      <c r="G34" s="17" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
@@ -11629,7 +11657,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G35" s="11" t="n">
+      <c r="G35" s="17" t="n">
         <v>46285</v>
       </c>
     </row>
@@ -11656,11 +11684,17 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Export operational reports and maintain a tenant backup path without flattening audit history.</t>
-        </is>
-      </c>
-      <c r="F36" s="12" t="inlineStr"/>
-      <c r="G36" s="11" t="n"/>
+          <t>Generate a date-range monthly PDF with revenue, sales-origin, procurement, production and inventory charts and tables, alongside exports and a tenant backup.</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="G36" s="17" t="n">
+        <v>46290</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
@@ -11689,7 +11723,7 @@
         </is>
       </c>
       <c r="F37" s="12" t="inlineStr"/>
-      <c r="G37" s="11" t="n"/>
+      <c r="G37" s="17" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="12" t="inlineStr">
@@ -11722,7 +11756,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G38" s="11" t="n">
+      <c r="G38" s="17" t="n">
         <v>46285</v>
       </c>
     </row>
@@ -11757,7 +11791,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G39" s="11" t="n">
+      <c r="G39" s="17" t="n">
         <v>46285</v>
       </c>
     </row>
@@ -11792,7 +11826,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G40" s="11" t="n">
+      <c r="G40" s="17" t="n">
         <v>46289</v>
       </c>
     </row>
@@ -11827,7 +11861,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G41" s="11" t="n">
+      <c r="G41" s="17" t="n">
         <v>46285</v>
       </c>
     </row>
@@ -11862,7 +11896,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G42" s="11" t="n">
+      <c r="G42" s="17" t="n">
         <v>46285</v>
       </c>
     </row>
@@ -11897,7 +11931,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G43" s="11" t="n">
+      <c r="G43" s="17" t="n">
         <v>46286</v>
       </c>
     </row>
@@ -11932,7 +11966,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G44" s="11" t="n">
+      <c r="G44" s="17" t="n">
         <v>46289</v>
       </c>
     </row>
@@ -11967,7 +12001,7 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="G45" s="11" t="n">
+      <c r="G45" s="17" t="n">
         <v>46290</v>
       </c>
     </row>

</xml_diff>